<commit_message>
Added tags to the rest of the pages in the documentation category and improved the wording slightly
</commit_message>
<xml_diff>
--- a/docu-content/010_Documentation/200_Terminology/SortedList_of_Terms.xlsx
+++ b/docu-content/010_Documentation/200_Terminology/SortedList_of_Terms.xlsx
@@ -1,19 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aklep\WebstormProjects\Freon-documentation\docu-content\010_Documentation\200_Terminology\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{524FC67F-DE2F-428C-85E0-D26EB10BC029}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{51154000-4CF9-4945-B87D-6262E1C33001}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{DB8CC088-8583-4FF2-9A6E-2F9270EA0E65}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" activeTab="1" xr2:uid="{DB8CC088-8583-4FF2-9A6E-2F9270EA0E65}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -25,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="120">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="528" uniqueCount="491">
   <si>
     <t>named property projection</t>
   </si>
@@ -346,6 +347,1073 @@
   </si>
   <si>
     <t>declared nodes</t>
+  </si>
+  <si>
+    <t>parent nodes</t>
+  </si>
+  <si>
+    <t>All named nodes that are visible in the parent namespace of this namespace.</t>
+  </si>
+  <si>
+    <t>imported nodes</t>
+  </si>
+  <si>
+    <t>alternative nodes</t>
+  </si>
+  <si>
+    <t>visible nodes</t>
+  </si>
+  <si>
+    <t>All named nodes that are accessible/visible/usable within this namespace, which is build based on the declared nodes, parent nodes, imported and alternatives nodes.</t>
+  </si>
+  <si>
+    <t>private property</t>
+  </si>
+  <si>
+    <t>public property</t>
+  </si>
+  <si>
+    <t>The principle that roughly 80% of the effects come from 20% of the causes; used in Freon to explain how the framework focuses on simplifying the majority of language-engineering tasks.</t>
+  </si>
+  <si>
+    <t>Abstract Syntax Tree (AST)</t>
+  </si>
+  <si>
+    <t>Automatic restructuring of binary expression trees in Freon so that operator precedence is reflected correctly after editing.</t>
+  </si>
+  <si>
+    <t>Embedding Freon</t>
+  </si>
+  <si>
+    <t>Integrating the Freon editor into a custom web application, typically using Svelte components.</t>
+  </si>
+  <si>
+    <t>FreNodeReference</t>
+  </si>
+  <si>
+    <t>A Freon class that represents name-based references, ensuring models remain trees instead of graphs.</t>
+  </si>
+  <si>
+    <t>Freon</t>
+  </si>
+  <si>
+    <t>The Freon framework for building DSL editors for the web; also the Frisian word for “friend.”</t>
+  </si>
+  <si>
+    <t>Freon interpreter framework</t>
+  </si>
+  <si>
+    <t>A Freon runtime framework that allows execution or simulation of DSL models.</t>
+  </si>
+  <si>
+    <t>LionWeb</t>
+  </si>
+  <si>
+    <t>An open initiative for web-based interoperability of modeling tools using a standard JSON interchange format.</t>
+  </si>
+  <si>
+    <t>LionWeb repository</t>
+  </si>
+  <si>
+    <t>A server implementation that stores models using the LionWeb protocol; can be connected to Freon for model persistence.</t>
+  </si>
+  <si>
+    <t>Model unit</t>
+  </si>
+  <si>
+    <t>A modular part of a model that can be edited or stored separately, enabling large-scale DSL models.</t>
+  </si>
+  <si>
+    <t>Name-based reference</t>
+  </si>
+  <si>
+    <t>A Freon reference mechanism that identifies model elements by name rather than by internal ID.</t>
+  </si>
+  <si>
+    <t>Object Constraint Language (OCL)</t>
+  </si>
+  <si>
+    <t>A formal language co-created by Jos Warmer for expressing constraints on UML models.</t>
+  </si>
+  <si>
+    <t>Pareto principle</t>
+  </si>
+  <si>
+    <t>Projection</t>
+  </si>
+  <si>
+    <t>The visual representation of the model’s AST displayed and manipulated in the Freon editor.</t>
+  </si>
+  <si>
+    <t>Projectional editing</t>
+  </si>
+  <si>
+    <t>An editing paradigm where users work directly on the model structure (AST) instead of plain text.</t>
+  </si>
+  <si>
+    <t>Fre-tools</t>
+  </si>
+  <si>
+    <t>The modular components generated by Freon, such as the editor, scoper, typer, validator, parser, and standard library.</t>
+  </si>
+  <si>
+    <t>Stacked Architecture</t>
+  </si>
+  <si>
+    <t>Freon’s three-level structure combining default, definition-based, and custom code layers.</t>
+  </si>
+  <si>
+    <t>Customization Level</t>
+  </si>
+  <si>
+    <t>The layer where handwritten TypeScript code extends or replaces generated behavior in Freon.</t>
+  </si>
+  <si>
+    <t>Box Provider</t>
+  </si>
+  <si>
+    <t>A generated class that produces boxes for specific AST concepts in the Freon editor.</t>
+  </si>
+  <si>
+    <t>Custom Projection</t>
+  </si>
+  <si>
+    <t>A user-defined method that returns a box for a given concept, registered in nodeTypeToBoxMethod.</t>
+  </si>
+  <si>
+    <t>Custom Action</t>
+  </si>
+  <si>
+    <t>A user-defined editor action created with FreCustomAction.create().</t>
+  </si>
+  <si>
+    <t>Projection Priority</t>
+  </si>
+  <si>
+    <t>The Freon mechanism that determines whether a projection comes from a custom, definition-based, or default source.</t>
+  </si>
+  <si>
+    <t>FreProjectionHandler</t>
+  </si>
+  <si>
+    <t>Box Role</t>
+  </si>
+  <si>
+    <t>External Component</t>
+  </si>
+  <si>
+    <t>A Svelte or Svelte-wrapped component embedded inside a Freon projection.</t>
+  </si>
+  <si>
+    <t>RenderComponent</t>
+  </si>
+  <si>
+    <t>Freon’s internal renderer that displays a childBox inside an external component.</t>
+  </si>
+  <si>
+    <t>FreComponentProps</t>
+  </si>
+  <si>
+    <t>The properties passed to an external component, containing editor and box references.</t>
+  </si>
+  <si>
+    <t>Box API</t>
+  </si>
+  <si>
+    <t>Key editor box methods such as findParam(), setFocus(), and refreshComponent().</t>
+  </si>
+  <si>
+    <t>FreScoper Interface</t>
+  </si>
+  <si>
+    <t>Custom Scoper</t>
+  </si>
+  <si>
+    <t>FreTyper Interface</t>
+  </si>
+  <si>
+    <t>Custom Typer</t>
+  </si>
+  <si>
+    <t>FreReader Interface</t>
+  </si>
+  <si>
+    <t>FreWriter Interface</t>
+  </si>
+  <si>
+    <t>FreStdlib Interface</t>
+  </si>
+  <si>
+    <t>Singleton Pattern</t>
+  </si>
+  <si>
+    <t>Ensures only one instance of the standard library (stdlib) exists at runtime.</t>
+  </si>
+  <si>
+    <t>Abstract concept</t>
+  </si>
+  <si>
+    <t>A concept that cannot be instantiated directly; other concepts inherit from it.</t>
+  </si>
+  <si>
+    <t>Binary expression</t>
+  </si>
+  <si>
+    <t>Boolean type</t>
+  </si>
+  <si>
+    <t>A primitive type with two values: true or false.</t>
+  </si>
+  <si>
+    <t>Concept</t>
+  </si>
+  <si>
+    <t>The primary building block of a Freon metamodel, similar to a class in UML.</t>
+  </si>
+  <si>
+    <t>Editor definition (.edit)</t>
+  </si>
+  <si>
+    <t>GradeScore</t>
+  </si>
+  <si>
+    <t>A concept representing a grading rule composed of a grade and an expression.</t>
+  </si>
+  <si>
+    <t>Limited concept</t>
+  </si>
+  <si>
+    <t>Metamodel</t>
+  </si>
+  <si>
+    <t>The structure that defines the syntax and semantics of a DSL in Freon.</t>
+  </si>
+  <si>
+    <t>Namespace addition</t>
+  </si>
+  <si>
+    <t>A rule allowing one namespace to import names from another (e.g., from a related page).</t>
+  </si>
+  <si>
+    <t>Projectional editor</t>
+  </si>
+  <si>
+    <t>An editor that directly manipulates the AST, ensuring models are always syntactically valid.</t>
+  </si>
+  <si>
+    <t>Reference</t>
+  </si>
+  <si>
+    <t>A property linking one concept to another (similar to associations in UML).</t>
+  </si>
+  <si>
+    <t>Reference shortcut</t>
+  </si>
+  <si>
+    <t>A shortcut allowing automatic creation of reference nodes without double selection.</t>
+  </si>
+  <si>
+    <t>Scope (.scope)</t>
+  </si>
+  <si>
+    <t>A file that defines namespaces and visibility rules for model elements.</t>
+  </si>
+  <si>
+    <t>Scoping</t>
+  </si>
+  <si>
+    <t>The mechanism that determines which names or elements are visible in a certain context.</t>
+  </si>
+  <si>
+    <t>Typing</t>
+  </si>
+  <si>
+    <t>Determines which elements are valid in specific locations within a model or Abstract Syntax Tree (AST).</t>
+  </si>
+  <si>
+    <t>Validation</t>
+  </si>
+  <si>
+    <t>Defines the rules that must hold in a language beyond syntax level, ensuring consistency and correctness of the model.</t>
+  </si>
+  <si>
+    <t>Scoping, Typing, and Validation</t>
+  </si>
+  <si>
+    <t>The three main components of Freon’s semantic analysis framework.</t>
+  </si>
+  <si>
+    <t>Type Provider (Typer)</t>
+  </si>
+  <si>
+    <t>A definition (.type) file that specifies typing rules for a language.</t>
+  </si>
+  <si>
+    <t>Type Concept</t>
+  </si>
+  <si>
+    <t>Declares which AST concepts are recognized as types.</t>
+  </si>
+  <si>
+    <t>hasType Rule</t>
+  </si>
+  <si>
+    <t>Identifies which AST concepts or interfaces have an associated type.</t>
+  </si>
+  <si>
+    <t>Inference Rule</t>
+  </si>
+  <si>
+    <t>Defines how to determine the type of a term, e.g. infertype self.declaredType.</t>
+  </si>
+  <si>
+    <t>FreType Interface</t>
+  </si>
+  <si>
+    <t>Anytype Rule</t>
+  </si>
+  <si>
+    <t>Type Comparison</t>
+  </si>
+  <si>
+    <t>Type concept instances cannot be compared by identity; comparison must use equalsto or conformsto.</t>
+  </si>
+  <si>
+    <t>Validator Definition</t>
+  </si>
+  <si>
+    <t>A .valid file containing the validation rules applied to models built by the user.</t>
+  </si>
+  <si>
+    <t>Validation Rules</t>
+  </si>
+  <si>
+    <t>Simple Value Rule</t>
+  </si>
+  <si>
+    <t>Restricts a property to specific values or numeric ranges.</t>
+  </si>
+  <si>
+    <t>Valid Identifier Rule</t>
+  </si>
+  <si>
+    <t>Checks whether identifiers follow TypeScript’s identifier rules (validIdentifier).</t>
+  </si>
+  <si>
+    <t>Type Check Rule</t>
+  </si>
+  <si>
+    <t>Verifies that two elements have compatible or identical types (typecheck equalsType or typecheck conformsTo).</t>
+  </si>
+  <si>
+    <t>Custom Message Rule</t>
+  </si>
+  <si>
+    <t>Default Validation Rules</t>
+  </si>
+  <si>
+    <t>Automatically enforced checks such as required properties, valid references, and non-empty lists.</t>
+  </si>
+  <si>
+    <t>Severity Levels</t>
+  </si>
+  <si>
+    <t>Possible values for validation message severity: error, warning, hint, improvement, todo, and info.</t>
+  </si>
+  <si>
+    <t>freon type-it</t>
+  </si>
+  <si>
+    <t>freon validate-it</t>
+  </si>
+  <si>
+    <t>freon all</t>
+  </si>
+  <si>
+    <t>Freon Editor</t>
+  </si>
+  <si>
+    <t>AST.change()</t>
+  </si>
+  <si>
+    <t>A helper method from @freon4dsl/core to ensure all model mutations are MobX-reactive.</t>
+  </si>
+  <si>
+    <t>MobX Reactivity</t>
+  </si>
+  <si>
+    <t>The reactive data layer used in Freon to track model state and automatically update the UI.</t>
+  </si>
+  <si>
+    <t>FreUndoManager</t>
+  </si>
+  <si>
+    <t>Component that handles undo and redo operations for model edits.</t>
+  </si>
+  <si>
+    <t>initialize()</t>
+  </si>
+  <si>
+    <t>Function used in external components to set up and synchronize data before rendering.</t>
+  </si>
+  <si>
+    <t>Interpreter Framework</t>
+  </si>
+  <si>
+    <t>Freon’s subsystem that enables the evaluation of DSL models directly from their Abstract Syntax Tree (AST).</t>
+  </si>
+  <si>
+    <t>Interpreter</t>
+  </si>
+  <si>
+    <t>Evaluation</t>
+  </si>
+  <si>
+    <t>The process of computing the value associated with an AST node during interpretation.</t>
+  </si>
+  <si>
+    <t>Evaluation Function</t>
+  </si>
+  <si>
+    <t>A generated or user-defined method that determines the meaning or output of a specific AST node.</t>
+  </si>
+  <si>
+    <t>Interpreter Context</t>
+  </si>
+  <si>
+    <t>A runtime data structure that stores variable bindings, constants, and references during evaluation, allowing nested evaluations to access local and parent scopes.</t>
+  </si>
+  <si>
+    <t>Runtime Object (RtObject)</t>
+  </si>
+  <si>
+    <t>The base class for all runtime results produced by interpretation, ensuring a clear separation between model and runtime layers.</t>
+  </si>
+  <si>
+    <t>M2 Level</t>
+  </si>
+  <si>
+    <t>The language definition level, describing available concepts in .ast files.</t>
+  </si>
+  <si>
+    <t>M1 Level</t>
+  </si>
+  <si>
+    <t>The model level, containing user-created instances of language concepts edited in the Freon editor.</t>
+  </si>
+  <si>
+    <t>M0 Level</t>
+  </si>
+  <si>
+    <t>The runtime level, representing values or results from executing or interpreting M1 models.</t>
+  </si>
+  <si>
+    <t>Meta Levels</t>
+  </si>
+  <si>
+    <t>The conceptual separation of model definition (M2), model instance (M1), and runtime execution (M0).</t>
+  </si>
+  <si>
+    <t>Operator Priority</t>
+  </si>
+  <si>
+    <t>Runtime Object Library</t>
+  </si>
+  <si>
+    <t>A collection of classes used for representing evaluated runtime values.</t>
+  </si>
+  <si>
+    <t>RtNumber</t>
+  </si>
+  <si>
+    <t>Represents numeric values at runtime.</t>
+  </si>
+  <si>
+    <t>RtString</t>
+  </si>
+  <si>
+    <t>Represents string values.</t>
+  </si>
+  <si>
+    <t>RtBoolean</t>
+  </si>
+  <si>
+    <t>Represents boolean values.</t>
+  </si>
+  <si>
+    <t>RtArray</t>
+  </si>
+  <si>
+    <t>Represents arrays of runtime objects.</t>
+  </si>
+  <si>
+    <t>RtError</t>
+  </si>
+  <si>
+    <t>Represents runtime errors encountered during interpretation.</t>
+  </si>
+  <si>
+    <t>Domain-Specific Runtime Class</t>
+  </si>
+  <si>
+    <t>A subclass of RtObject that models domain-specific runtime behavior.</t>
+  </si>
+  <si>
+    <t>Parameter Lookup</t>
+  </si>
+  <si>
+    <t>The process by which the interpreter retrieves a parameter’s current value from the active context.</t>
+  </si>
+  <si>
+    <t>Evaluation Override</t>
+  </si>
+  <si>
+    <t>The act of redefining a generated evaluation function to perform actual interpretation logic.</t>
+  </si>
+  <si>
+    <t>AST-Based Interpretation</t>
+  </si>
+  <si>
+    <t>Evaluation performed directly on the AST, without parsing or lexing steps, thanks to Freon’s projectional editor.</t>
+  </si>
+  <si>
+    <t>Partial Interpretation</t>
+  </si>
+  <si>
+    <t>Occurs when evaluation cannot be completed because required context or values are missing.</t>
+  </si>
+  <si>
+    <t>Concrete Syntax Tree (CST)</t>
+  </si>
+  <si>
+    <t>A tree representing how a model appears visually; in Freon, this corresponds to the Box Model.</t>
+  </si>
+  <si>
+    <t>Box Tree</t>
+  </si>
+  <si>
+    <t>The hierarchy of boxes used by the Freon editor to represent layout and structure of a model on screen.</t>
+  </si>
+  <si>
+    <t>Svelte Components</t>
+  </si>
+  <si>
+    <t>UI building blocks written in Svelte; used to extend or replace parts of Freon’s editor interface.</t>
+  </si>
+  <si>
+    <t>Document Object Model (DOM)</t>
+  </si>
+  <si>
+    <t>The browser’s structure of HTML elements; Freon’s rendered boxes eventually map to DOM nodes.</t>
+  </si>
+  <si>
+    <t>Editor Framework</t>
+  </si>
+  <si>
+    <t>The set of Freon subsystems that manage projections, actions, caret movement, and rendering.</t>
+  </si>
+  <si>
+    <t>Triggers and Key Bindings</t>
+  </si>
+  <si>
+    <t>User input patterns (keyboard or mouse) that activate specific editor actions.</t>
+  </si>
+  <si>
+    <t>Caret Position</t>
+  </si>
+  <si>
+    <t>The current insertion point in the editor, managed by the FreCaret interface.</t>
+  </si>
+  <si>
+    <t>Freon Language Workbench</t>
+  </si>
+  <si>
+    <t>The Freon platform for defining, generating, and executing web-based DSL editors.</t>
+  </si>
+  <si>
+    <t>The base interface for all Freon model elements, providing identity and structural information.</t>
+  </si>
+  <si>
+    <t>FreAction</t>
+  </si>
+  <si>
+    <t>Defines an executable editor operation such as inserting, deleting, or modifying nodes.</t>
+  </si>
+  <si>
+    <t>FreCustomAction</t>
+  </si>
+  <si>
+    <t>User-defined action class used to add or override default editor behavior.</t>
+  </si>
+  <si>
+    <t>FreBehavior</t>
+  </si>
+  <si>
+    <t>Encapsulates user interaction logic that links triggers to editor actions.</t>
+  </si>
+  <si>
+    <t>FreEditor</t>
+  </si>
+  <si>
+    <t>The main runtime editor interface controlling projections, boxes, and user interactions.</t>
+  </si>
+  <si>
+    <t>FreCaret</t>
+  </si>
+  <si>
+    <t>Interface representing the caret’s current position, movement, and focus behavior.</t>
+  </si>
+  <si>
+    <t>FrePostAction</t>
+  </si>
+  <si>
+    <t>Action executed after a primary action, often for cleanup or UI refresh.</t>
+  </si>
+  <si>
+    <t>FreTriggerType</t>
+  </si>
+  <si>
+    <t>Enumeration defining input types (e.g., key, mouse) that can trigger editor actions.</t>
+  </si>
+  <si>
+    <t>FreTriggerUse</t>
+  </si>
+  <si>
+    <t>Enumeration describing how triggers are applied (e.g., pressed, released, repeated).</t>
+  </si>
+  <si>
+    <t>Container Descriptor (piContainer)</t>
+  </si>
+  <si>
+    <t>Metadata linking an element to its parent container in the AST hierarchy.</t>
+  </si>
+  <si>
+    <t>Alternative Nodes</t>
+  </si>
+  <si>
+    <t>Declared nodes from namespaces that have an alternative relationship with the current namespace, defined in the alternatives block.</t>
+  </si>
+  <si>
+    <t>Declared Nodes</t>
+  </si>
+  <si>
+    <t>Imported Nodes</t>
+  </si>
+  <si>
+    <t>Declared nodes of other namespaces included via an imports block; private properties are excluded.</t>
+  </si>
+  <si>
+    <t>Namespace</t>
+  </si>
+  <si>
+    <t>Namespace Graph / Tree</t>
+  </si>
+  <si>
+    <t>The overall structure formed by all namespaces; forms a tree when hierarchical, or a directed graph when imports or alternatives exist.</t>
+  </si>
+  <si>
+    <t>Parent Nodes</t>
+  </si>
+  <si>
+    <t>Visible nodes inherited from the parent namespace, contributing to hierarchical or lexical scoping.</t>
+  </si>
+  <si>
+    <t>Private Properties</t>
+  </si>
+  <si>
+    <t>Properties in .ast files marked with the private keyword; visible only within their own namespace, not when imported elsewhere.</t>
+  </si>
+  <si>
+    <t>Visible Nodes</t>
+  </si>
+  <si>
+    <t>The complete set of named nodes accessible in a namespace, constructed from declared, imported, alternative, and parent nodes.</t>
+  </si>
+  <si>
+    <t>alternatives (keyword)</t>
+  </si>
+  <si>
+    <t>Defines replacement or non-hierarchical visibility relationships between namespaces.</t>
+  </si>
+  <si>
+    <t>imports (keyword)</t>
+  </si>
+  <si>
+    <t>Adds declared nodes from other namespaces to the current namespace’s visible nodes; can be marked recursive.</t>
+  </si>
+  <si>
+    <t>isNamespace (keyword)</t>
+  </si>
+  <si>
+    <t>Declares which concepts, model units, or interfaces identify namespaces within the language.</t>
+  </si>
+  <si>
+    <t>private (keyword)</t>
+  </si>
+  <si>
+    <t>Marks properties in .ast files that should not be imported into other namespaces.</t>
+  </si>
+  <si>
+    <t>self (keyword)</t>
+  </si>
+  <si>
+    <t>Optional prefix for referencing direct properties within scoping expressions, similar to “this” in programming languages.</t>
+  </si>
+  <si>
+    <t>if(MetaType) (function)</t>
+  </si>
+  <si>
+    <t>Limits a scope expression to nodes of a specific metatype (concept or model unit); skips others.</t>
+  </si>
+  <si>
+    <t>owner() (function)</t>
+  </si>
+  <si>
+    <t>Returns the owning namespace of the current property or node, used for navigating upward through the AST.</t>
+  </si>
+  <si>
+    <t>type() (function)</t>
+  </si>
+  <si>
+    <t>Returns the type of a node as determined by the typer; must appear at the end of an expression.</t>
+  </si>
+  <si>
+    <t>Interface defining how a language concept is visually projected in the editor.</t>
+  </si>
+  <si>
+    <t>Base interface for all expression elements in the Freon model.</t>
+  </si>
+  <si>
+    <t>Custom Box Definitions</t>
+  </si>
+  <si>
+    <t>User-defined layouts or components replacing generated box structures.</t>
+  </si>
+  <si>
+    <t>The precedence rules defining how binary expressions are grouped during editing and interpretation.</t>
+  </si>
+  <si>
+    <t>FreEnvironment</t>
+  </si>
+  <si>
+    <t>Central registry providing access to language definitions, scopers, typers, and validators.</t>
+  </si>
+  <si>
+    <t>FreScoper</t>
+  </si>
+  <si>
+    <t>FreValidator</t>
+  </si>
+  <si>
+    <t>FreTyper</t>
+  </si>
+  <si>
+    <t>FreTyperPart</t>
+  </si>
+  <si>
+    <t>A modular part of the typer that implements type inference for a subset of concepts.</t>
+  </si>
+  <si>
+    <t>FreReader</t>
+  </si>
+  <si>
+    <t>Component that parses models from text or serialized data into AST structures.</t>
+  </si>
+  <si>
+    <t>FreWriter</t>
+  </si>
+  <si>
+    <t>Component that serializes models back to text or persistent form.</t>
+  </si>
+  <si>
+    <t>FreStdlib</t>
+  </si>
+  <si>
+    <t>Language Environment</t>
+  </si>
+  <si>
+    <t>Runtime environment containing the generated Fre-tools for a specific language.</t>
+  </si>
+  <si>
+    <t>Scoping Rules</t>
+  </si>
+  <si>
+    <t>Definitions determining which names are visible and resolvable in a given context.</t>
+  </si>
+  <si>
+    <t>Name Resolution</t>
+  </si>
+  <si>
+    <t>Process of linking references in the model to their declared elements.</t>
+  </si>
+  <si>
+    <t>Rules that check whether models obey the domain semantics of a language.</t>
+  </si>
+  <si>
+    <t>Error Severity</t>
+  </si>
+  <si>
+    <t>Classification of validation messages (e.g., error, warning, hint, info).</t>
+  </si>
+  <si>
+    <t>Type Inference</t>
+  </si>
+  <si>
+    <t>Process of determining the type of a model element based on context and rules.</t>
+  </si>
+  <si>
+    <t>Type Equality</t>
+  </si>
+  <si>
+    <t>Rules defining when two types are considered identical within the type system.</t>
+  </si>
+  <si>
+    <t>Type Conformance</t>
+  </si>
+  <si>
+    <t>Rules defining whether one type can be used where another is expected.</t>
+  </si>
+  <si>
+    <t>Parsing (Reader)</t>
+  </si>
+  <si>
+    <t>The operation of reading a textual or serialized representation into a Freon model.</t>
+  </si>
+  <si>
+    <t>Unparsing (Writer)</t>
+  </si>
+  <si>
+    <t>The reverse process of serializing a model from AST to text.</t>
+  </si>
+  <si>
+    <t>Standard Library (Stdlib)</t>
+  </si>
+  <si>
+    <t>Collection of built-in elements and reusable constructs defined for a language.</t>
+  </si>
+  <si>
+    <t>Named Elements</t>
+  </si>
+  <si>
+    <t>Model elements with unique names that can be referenced by other parts of the model.</t>
+  </si>
+  <si>
+    <t>The internal tree structure of a model, where each node represents an instance of a language concept. It is the core model manipulated directly by users of the Freon editor instead of plain text.</t>
+  </si>
+  <si>
+    <t>See Abstract Syntax Tree (AST).</t>
+  </si>
+  <si>
+    <t>Balancing expressions</t>
+  </si>
+  <si>
+    <t>An identifier assigned to a box that links it to specific editor behaviors or actions. Box roles connect visual elements in a projection to the logic that handles user interactions.</t>
+  </si>
+  <si>
+    <r>
+      <t>Definition of user-defined error messages and severity levels (</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>message</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>severity</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>) used during validation.</t>
+    </r>
+  </si>
+  <si>
+    <t>A programming or modeling language tailored to a specific problem domain, providing constructs and abstractions closely aligned with domain concepts rather than general-purpose computation. In Freon, DSLs are designed, edited, and executed using generated tools that combine structural definitions (metamodels), projections, and validation rules.</t>
+  </si>
+  <si>
+    <t>Domain-Specific Language (DSL)</t>
+  </si>
+  <si>
+    <t>DSL</t>
+  </si>
+  <si>
+    <t>See Domain-Specific Language</t>
+  </si>
+  <si>
+    <t>Command that generates all dependent components in the correct order, ensuring compilable and consistent output.</t>
+  </si>
+  <si>
+    <t>Command that generates typing code from .type definition files.</t>
+  </si>
+  <si>
+    <t>Command that generates validation code from .valid definition files.</t>
+  </si>
+  <si>
+    <t>The .edit file section listing available external components in a language, and settings to be applied globally in the editor.</t>
+  </si>
+  <si>
+    <t>A general validation rule that applies to all concepts.</t>
+  </si>
+  <si>
+    <t>A subtype of Expression that defines an expression with a left and right operand, combined using an operator such as +, *, AND, or &gt;.</t>
+  </si>
+  <si>
+    <t>A subtype of Concept that defines a construct that produces a value.</t>
+  </si>
+  <si>
+    <t>freon scope-it</t>
+  </si>
+  <si>
+    <t>Command that generates scoping code from .scope definition files.</t>
+  </si>
+  <si>
+    <t>freon edit-it</t>
+  </si>
+  <si>
+    <t>Command that generates projection code from .edit definition files.</t>
+  </si>
+  <si>
+    <t>Command that generates code for all concepts, units etc. from .lang definition files.</t>
+  </si>
+  <si>
+    <t>freon ast-it</t>
+  </si>
+  <si>
+    <t>freon parse-it</t>
+  </si>
+  <si>
+    <t>Command that generates parser code  from .edit definition files.</t>
+  </si>
+  <si>
+    <t>Command that generates UML diagrams  from .ast definition files.</t>
+  </si>
+  <si>
+    <t>freon diagram-it</t>
+  </si>
+  <si>
+    <t>freon interpret-it</t>
+  </si>
+  <si>
+    <t>Command that generates interpreter code  for your language.</t>
+  </si>
+  <si>
+    <t>freon clean-it</t>
+  </si>
+  <si>
+    <t>Command that removes all generated TypeScript code for your language.</t>
+  </si>
+  <si>
+    <t>FreProjection Interface</t>
+  </si>
+  <si>
+    <t>Interface defining  how models are parsed from text input into Freon’s AST representation.</t>
+  </si>
+  <si>
+    <t>Interface defining  the logic for resolving references and visible names within a Freon model.</t>
+  </si>
+  <si>
+    <t>Interface defining  all predefined instances and limited concepts for a given language in Freon.</t>
+  </si>
+  <si>
+    <t>Interface defining  the logic for type inference, type equality, and conformance checks.</t>
+  </si>
+  <si>
+    <t>Interface defining  how models are serialized or exported from Freon to text or files.</t>
+  </si>
+  <si>
+    <t>FreError Interface</t>
+  </si>
+  <si>
+    <t>Interface defining issues or diagnostics produced during validation or typing.</t>
+  </si>
+  <si>
+    <t>FreExpression Interface</t>
+  </si>
+  <si>
+    <t>FreNamedNode Interface</t>
+  </si>
+  <si>
+    <t>FreNode Interface</t>
+  </si>
+  <si>
+    <t>Interface that extends FreNode with a name property used in references and scoping.</t>
+  </si>
+  <si>
+    <t>The projectional graphical editor generated from a Freon DSL specification.</t>
+  </si>
+  <si>
+    <t>A Freon runtime class that manages projection rendering and links between AST nodes and visual boxes.</t>
+  </si>
+  <si>
+    <t>Component responsible for resolving references and managing name visibility in the model.</t>
+  </si>
+  <si>
+    <t>Component that holds the standard library of predefined elements and limited concepts available in a language.</t>
+  </si>
+  <si>
+    <t>Interface implemented by all type concepts in Freon.</t>
+  </si>
+  <si>
+    <t>Component for inferring and checking the types of model elements.</t>
+  </si>
+  <si>
+    <t>Component for validating models to ensure semantic correctness.</t>
+  </si>
+  <si>
+    <t>FreValidator Interface</t>
+  </si>
+  <si>
+    <t>Interface defining how models are validated to ensure semantic correctness.</t>
+  </si>
+  <si>
+    <t>Global section</t>
+  </si>
+  <si>
+    <r>
+      <t>All declared nodes from other namespaces that have an </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>alternative relationship</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t> with this namespace.</t>
+    </r>
   </si>
   <si>
     <r>
@@ -354,7 +1422,7 @@
     <r>
       <rPr>
         <sz val="9.9"/>
-        <color rgb="FF080808"/>
+        <color rgb="FFFF0000"/>
         <rFont val="Consolas"/>
         <family val="3"/>
       </rPr>
@@ -363,7 +1431,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FF080808"/>
+        <color rgb="FFFF0000"/>
         <rFont val="Arial"/>
         <family val="2"/>
       </rPr>
@@ -373,7 +1441,7 @@
       <rPr>
         <i/>
         <sz val="11"/>
-        <color rgb="FF080808"/>
+        <color rgb="FFFF0000"/>
         <rFont val="Arial"/>
         <family val="2"/>
       </rPr>
@@ -382,21 +1450,12 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FF080808"/>
+        <color rgb="FFFF0000"/>
         <rFont val="Arial"/>
         <family val="2"/>
       </rPr>
       <t>) in the namespace subtree.</t>
     </r>
-  </si>
-  <si>
-    <t>parent nodes</t>
-  </si>
-  <si>
-    <t>All named nodes that are visible in the parent namespace of this namespace.</t>
-  </si>
-  <si>
-    <t>imported nodes</t>
   </si>
   <si>
     <r>
@@ -406,7 +1465,7 @@
       <rPr>
         <i/>
         <sz val="11"/>
-        <color rgb="FF080808"/>
+        <color rgb="FFFF0000"/>
         <rFont val="Arial"/>
         <family val="2"/>
       </rPr>
@@ -415,48 +1474,12 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FF080808"/>
+        <color rgb="FFFF0000"/>
         <rFont val="Arial"/>
         <family val="2"/>
       </rPr>
       <t> with this namespace.</t>
     </r>
-  </si>
-  <si>
-    <t>alternative nodes</t>
-  </si>
-  <si>
-    <r>
-      <t>All declared nodes from other namespaces that have an </t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="11"/>
-        <color rgb="FF080808"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>alternative relationship</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF080808"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t> with this namespace.</t>
-    </r>
-  </si>
-  <si>
-    <t>visible nodes</t>
-  </si>
-  <si>
-    <t>All named nodes that are accessible/visible/usable within this namespace, which is build based on the declared nodes, parent nodes, imported and alternatives nodes.</t>
-  </si>
-  <si>
-    <t>private property</t>
   </si>
   <si>
     <r>
@@ -466,7 +1489,7 @@
       <rPr>
         <i/>
         <sz val="11"/>
-        <color rgb="FF080808"/>
+        <color rgb="FFFF0000"/>
         <rFont val="Arial"/>
         <family val="2"/>
       </rPr>
@@ -475,15 +1498,12 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FF080808"/>
+        <color rgb="FFFF0000"/>
         <rFont val="Arial"/>
         <family val="2"/>
       </rPr>
       <t> be included in the visible nodes of a namespace when the namespace in which it is declared is imported, using namespace imports.</t>
     </r>
-  </si>
-  <si>
-    <t>public property</t>
   </si>
   <si>
     <r>
@@ -492,7 +1512,7 @@
     <r>
       <rPr>
         <sz val="9.9"/>
-        <color rgb="FF080808"/>
+        <color rgb="FFFF0000"/>
         <rFont val="Consolas"/>
         <family val="3"/>
       </rPr>
@@ -501,19 +1521,211 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FF080808"/>
+        <color rgb="FFFF0000"/>
         <rFont val="Arial"/>
         <family val="2"/>
       </rPr>
       <t> with regard to namespace imports.</t>
     </r>
   </si>
+  <si>
+    <t>Action</t>
+  </si>
+  <si>
+    <t>Alternative namespace</t>
+  </si>
+  <si>
+    <t>A statement in the scoper definition that removes the names from the parent namespace, and replaces them by the names of another namespace.</t>
+  </si>
+  <si>
+    <t>Box</t>
+  </si>
+  <si>
+    <t>Box tree / box model</t>
+  </si>
+  <si>
+    <t>conformsto (keyword)</t>
+  </si>
+  <si>
+    <t>See Concrete Syntax Tree</t>
+  </si>
+  <si>
+    <t>A user-defined replacement for, or augmentation to, the generated scoper, currently applied globally rather than per concept.</t>
+  </si>
+  <si>
+    <t>A user-defined replacement for, or augmentation to, the generated typer, applied per concept.</t>
+  </si>
+  <si>
+    <t>All named nodes (with a name: identifier property) within a namespace’s AST subtree, including nodes that define other namespaces, but excluding the declared nodes from those namespaces.</t>
+  </si>
+  <si>
+    <t>A file describing how concepts and their properties are projected in the Freon editor, thus defining a projection set.</t>
+  </si>
+  <si>
+    <t>Editor</t>
+  </si>
+  <si>
+    <t>Enumeration</t>
+  </si>
+  <si>
+    <t>equalsto (keyword)</t>
+  </si>
+  <si>
+    <t>Expression (or Expression Concept)</t>
+  </si>
+  <si>
+    <t>Fragment</t>
+  </si>
+  <si>
+    <t>A component that traverses and evaluates the AST to compute values to be associated with certain nodes.</t>
+  </si>
+  <si>
+    <t>istype (keyword)</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Built-in validation rule ensuring that all elements in a list are unique, effectively treating the list as a strict set. Used in </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>.valid</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> files to enforce uniqueness constraints within Freon models.</t>
+    </r>
+  </si>
+  <si>
+    <t>isunique (keyword) / is-unique rule</t>
+  </si>
+  <si>
+    <t>Language engineer</t>
+  </si>
+  <si>
+    <t>Model</t>
+  </si>
+  <si>
+    <t>Named editor</t>
+  </si>
+  <si>
+    <t>Named property projection</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Built-in validation rule ensuring that lists are not empty. Used in </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>.valid</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> files to enforce that a property contains at least one element within a Freon model.</t>
+    </r>
+  </si>
+  <si>
+    <t>notempty (keyword) / not-empty rule</t>
+  </si>
+  <si>
+    <t>Precedence of projections</t>
+  </si>
+  <si>
+    <t>In a set of projections for the same concept, the priority of one projection over the other.</t>
+  </si>
+  <si>
+    <t>Projection set</t>
+  </si>
+  <si>
+    <t>Public property</t>
+  </si>
+  <si>
+    <t>Scope provider (or scoper)</t>
+  </si>
+  <si>
+    <t>A component that is able to determine for each term in the model which names of other elements of the model are visible.</t>
+  </si>
+  <si>
+    <t>Symbol</t>
+  </si>
+  <si>
+    <t>Term</t>
+  </si>
+  <si>
+    <t>Trigger</t>
+  </si>
+  <si>
+    <t>Type provider (or typer)</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">A specialized concept representing a type within a Freon language. It implements the </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>FreType</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> interface and is not part of the Abstract Syntax Tree (AST) itself but provides the type information associated with model elements or terms.</t>
+    </r>
+  </si>
+  <si>
+    <t>A component that is able to determine for each term in the model which type to associate with that term.</t>
+  </si>
+  <si>
+    <t>Typer</t>
+  </si>
+  <si>
+    <t>Typer file</t>
+  </si>
+  <si>
+    <t>User</t>
+  </si>
+  <si>
+    <t>Valid file</t>
+  </si>
+  <si>
+    <t>Validator</t>
+  </si>
+  <si>
+    <t>A component that is able to determine for each term in the model whether the term is correct or erroneous.</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5">
+  <fonts count="7">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -522,29 +1734,41 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <sz val="10"/>
-      <color rgb="FF0033B3"/>
+      <color theme="1"/>
+      <name val="Arial Unicode MS"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FFFF0000"/>
       <name val="JetBrains Mono"/>
       <family val="3"/>
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FF080808"/>
+      <color rgb="FFFF0000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
     <font>
       <sz val="9.9"/>
-      <color rgb="FF080808"/>
+      <color rgb="FFFF0000"/>
       <name val="Consolas"/>
       <family val="3"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF080808"/>
-      <name val="Arial"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="3">
@@ -588,26 +1812,49 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -925,7 +2172,7 @@
   <dimension ref="A1:B110"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="34.33203125" customWidth="1"/>
+    <col min="1" max="1" width="34.33203125" style="7" customWidth="1"/>
     <col min="2" max="2" width="86" style="2" customWidth="1"/>
   </cols>
   <sheetData>
@@ -933,10 +2180,10 @@
       <c r="A1" s="1"/>
     </row>
     <row r="2" spans="1:2" ht="27.6">
-      <c r="A2" s="4" t="s">
+      <c r="A2" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="3" t="s">
         <v>52</v>
       </c>
     </row>
@@ -944,37 +2191,37 @@
       <c r="A3" s="1"/>
     </row>
     <row r="4" spans="1:2">
-      <c r="A4" s="4" t="s">
+      <c r="A4" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B4" s="3" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="27.6">
-      <c r="A5" s="4" t="s">
+      <c r="A5" s="3" t="s">
         <v>95</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="B5" s="3" t="s">
         <v>96</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="28.2">
-      <c r="A6" s="4" t="s">
-        <v>112</v>
-      </c>
-      <c r="B6" s="4" t="s">
-        <v>113</v>
+      <c r="A6" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>442</v>
       </c>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="1"/>
     </row>
     <row r="8" spans="1:2">
-      <c r="A8" s="4" t="s">
+      <c r="A8" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="B8" s="3" t="s">
         <v>50</v>
       </c>
     </row>
@@ -982,10 +2229,10 @@
       <c r="A9" s="1"/>
     </row>
     <row r="10" spans="1:2">
-      <c r="A10" s="4" t="s">
+      <c r="A10" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="B10" s="4" t="s">
+      <c r="B10" s="3" t="s">
         <v>71</v>
       </c>
     </row>
@@ -993,10 +2240,10 @@
       <c r="A11" s="1"/>
     </row>
     <row r="12" spans="1:2">
-      <c r="A12" s="4" t="s">
+      <c r="A12" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="B12" s="4" t="s">
+      <c r="B12" s="3" t="s">
         <v>39</v>
       </c>
     </row>
@@ -1004,10 +2251,10 @@
       <c r="A13" s="1"/>
     </row>
     <row r="14" spans="1:2">
-      <c r="A14" s="4" t="s">
+      <c r="A14" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="B14" s="4" t="s">
+      <c r="B14" s="3" t="s">
         <v>97</v>
       </c>
     </row>
@@ -1015,10 +2262,10 @@
       <c r="A15" s="1"/>
     </row>
     <row r="16" spans="1:2">
-      <c r="A16" s="4" t="s">
+      <c r="A16" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="B16" s="4" t="s">
+      <c r="B16" s="3" t="s">
         <v>62</v>
       </c>
     </row>
@@ -1026,10 +2273,10 @@
       <c r="A17" s="1"/>
     </row>
     <row r="18" spans="1:2" ht="27.6">
-      <c r="A18" s="4" t="s">
+      <c r="A18" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="B18" s="4" t="s">
+      <c r="B18" s="3" t="s">
         <v>44</v>
       </c>
     </row>
@@ -1037,10 +2284,10 @@
       <c r="A19" s="1"/>
     </row>
     <row r="20" spans="1:2" ht="27.6">
-      <c r="A20" s="4" t="s">
+      <c r="A20" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="B20" s="4" t="s">
+      <c r="B20" s="3" t="s">
         <v>45</v>
       </c>
     </row>
@@ -1048,10 +2295,10 @@
       <c r="A21" s="1"/>
     </row>
     <row r="22" spans="1:2">
-      <c r="A22" s="4" t="s">
+      <c r="A22" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="B22" s="4" t="s">
+      <c r="B22" s="3" t="s">
         <v>46</v>
       </c>
     </row>
@@ -1059,10 +2306,10 @@
       <c r="A23" s="1"/>
     </row>
     <row r="24" spans="1:2">
-      <c r="A24" s="4" t="s">
+      <c r="A24" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="B24" s="4" t="s">
+      <c r="B24" s="3" t="s">
         <v>53</v>
       </c>
     </row>
@@ -1070,29 +2317,29 @@
       <c r="A25" s="1"/>
     </row>
     <row r="26" spans="1:2">
-      <c r="A26" s="4" t="s">
+      <c r="A26" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="B26" s="4" t="s">
+      <c r="B26" s="3" t="s">
         <v>54</v>
       </c>
     </row>
     <row r="27" spans="1:2" ht="28.2">
-      <c r="A27" s="4" t="s">
+      <c r="A27" s="3" t="s">
         <v>106</v>
       </c>
-      <c r="B27" s="4" t="s">
-        <v>107</v>
+      <c r="B27" s="3" t="s">
+        <v>443</v>
       </c>
     </row>
     <row r="28" spans="1:2">
       <c r="A28" s="1"/>
     </row>
     <row r="29" spans="1:2" ht="27.6">
-      <c r="A29" s="4" t="s">
+      <c r="A29" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="B29" s="4" t="s">
+      <c r="B29" s="3" t="s">
         <v>98</v>
       </c>
     </row>
@@ -1100,10 +2347,10 @@
       <c r="A30" s="1"/>
     </row>
     <row r="31" spans="1:2">
-      <c r="A31" s="4" t="s">
+      <c r="A31" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="B31" s="4" t="s">
+      <c r="B31" s="3" t="s">
         <v>67</v>
       </c>
     </row>
@@ -1111,10 +2358,10 @@
       <c r="A32" s="1"/>
     </row>
     <row r="33" spans="1:2">
-      <c r="A33" s="4" t="s">
+      <c r="A33" s="3" t="s">
         <v>64</v>
       </c>
-      <c r="B33" s="4" t="s">
+      <c r="B33" s="3" t="s">
         <v>65</v>
       </c>
     </row>
@@ -1122,10 +2369,10 @@
       <c r="A34" s="1"/>
     </row>
     <row r="35" spans="1:2" ht="27.6">
-      <c r="A35" s="4" t="s">
+      <c r="A35" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="B35" s="4" t="s">
+      <c r="B35" s="3" t="s">
         <v>55</v>
       </c>
     </row>
@@ -1133,10 +2380,10 @@
       <c r="A36" s="1"/>
     </row>
     <row r="37" spans="1:2">
-      <c r="A37" s="4" t="s">
+      <c r="A37" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="B37" s="4" t="s">
+      <c r="B37" s="3" t="s">
         <v>56</v>
       </c>
     </row>
@@ -1144,10 +2391,10 @@
       <c r="A38" s="1"/>
     </row>
     <row r="39" spans="1:2">
-      <c r="A39" s="4" t="s">
+      <c r="A39" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="B39" s="4" t="s">
+      <c r="B39" s="3" t="s">
         <v>57</v>
       </c>
     </row>
@@ -1155,37 +2402,37 @@
       <c r="A40" s="1"/>
     </row>
     <row r="41" spans="1:2">
-      <c r="A41" s="4" t="s">
+      <c r="A41" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="B41" s="4" t="s">
+      <c r="B41" s="3" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="42" spans="1:2" ht="27.6">
-      <c r="A42" s="4" t="s">
+      <c r="A42" s="3" t="s">
         <v>99</v>
       </c>
-      <c r="B42" s="4" t="s">
+      <c r="B42" s="3" t="s">
         <v>100</v>
       </c>
     </row>
     <row r="43" spans="1:2" ht="28.2">
-      <c r="A43" s="4" t="s">
-        <v>110</v>
-      </c>
-      <c r="B43" s="4" t="s">
-        <v>111</v>
+      <c r="A43" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="B43" s="3" t="s">
+        <v>444</v>
       </c>
     </row>
     <row r="44" spans="1:2">
       <c r="A44" s="1"/>
     </row>
     <row r="45" spans="1:2">
-      <c r="A45" s="4" t="s">
+      <c r="A45" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="B45" s="4" t="s">
+      <c r="B45" s="3" t="s">
         <v>80</v>
       </c>
     </row>
@@ -1193,10 +2440,10 @@
       <c r="A46" s="1"/>
     </row>
     <row r="47" spans="1:2" ht="27.6">
-      <c r="A47" s="4" t="s">
+      <c r="A47" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="B47" s="4" t="s">
+      <c r="B47" s="3" t="s">
         <v>83</v>
       </c>
     </row>
@@ -1204,10 +2451,10 @@
       <c r="A48" s="1"/>
     </row>
     <row r="49" spans="1:2" ht="27.6">
-      <c r="A49" s="4" t="s">
+      <c r="A49" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="B49" s="4" t="s">
+      <c r="B49" s="3" t="s">
         <v>78</v>
       </c>
     </row>
@@ -1215,374 +2462,374 @@
       <c r="A50" s="1"/>
     </row>
     <row r="51" spans="1:2" ht="15" thickBot="1">
-      <c r="A51" s="4" t="s">
+      <c r="A51" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="B51" s="4" t="s">
+      <c r="B51" s="3" t="s">
         <v>101</v>
       </c>
     </row>
     <row r="52" spans="1:2" ht="15" thickBot="1">
-      <c r="A52" s="5"/>
-      <c r="B52" s="6"/>
+      <c r="A52" s="4"/>
+      <c r="B52" s="5"/>
     </row>
     <row r="53" spans="1:2" ht="28.2" thickBot="1">
-      <c r="A53" s="3" t="s">
+      <c r="A53" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="B53" s="3" t="s">
+      <c r="B53" s="6" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="54" spans="1:2" ht="15" thickBot="1">
-      <c r="A54" s="5"/>
-      <c r="B54" s="6"/>
+      <c r="A54" s="4"/>
+      <c r="B54" s="5"/>
     </row>
     <row r="55" spans="1:2" ht="28.2" thickBot="1">
-      <c r="A55" s="3" t="s">
+      <c r="A55" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="B55" s="3" t="s">
+      <c r="B55" s="6" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="56" spans="1:2" ht="15" thickBot="1">
-      <c r="A56" s="5"/>
-      <c r="B56" s="6"/>
+      <c r="A56" s="4"/>
+      <c r="B56" s="5"/>
     </row>
     <row r="57" spans="1:2" ht="28.2" thickBot="1">
-      <c r="A57" s="3" t="s">
+      <c r="A57" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="B57" s="3" t="s">
+      <c r="B57" s="6" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="58" spans="1:2" ht="28.2" thickBot="1">
-      <c r="A58" s="3" t="s">
+      <c r="A58" s="6" t="s">
         <v>102</v>
       </c>
-      <c r="B58" s="3" t="s">
+      <c r="B58" s="6" t="s">
         <v>103</v>
       </c>
     </row>
     <row r="59" spans="1:2" ht="15" thickBot="1">
-      <c r="A59" s="5"/>
-      <c r="B59" s="6"/>
+      <c r="A59" s="4"/>
+      <c r="B59" s="5"/>
     </row>
     <row r="60" spans="1:2" ht="15" thickBot="1">
-      <c r="A60" s="5"/>
-      <c r="B60" s="6"/>
+      <c r="A60" s="4"/>
+      <c r="B60" s="5"/>
     </row>
     <row r="61" spans="1:2" ht="15" thickBot="1">
-      <c r="A61" s="3" t="s">
+      <c r="A61" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="B61" s="3" t="s">
+      <c r="B61" s="6" t="s">
         <v>74</v>
       </c>
     </row>
     <row r="62" spans="1:2" ht="15" thickBot="1">
-      <c r="A62" s="5"/>
-      <c r="B62" s="6"/>
+      <c r="A62" s="4"/>
+      <c r="B62" s="5"/>
     </row>
     <row r="63" spans="1:2" ht="15" thickBot="1">
-      <c r="A63" s="3" t="s">
+      <c r="A63" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="B63" s="3" t="s">
+      <c r="B63" s="6" t="s">
         <v>75</v>
       </c>
     </row>
     <row r="64" spans="1:2" ht="15" thickBot="1">
-      <c r="A64" s="5"/>
-      <c r="B64" s="6"/>
+      <c r="A64" s="4"/>
+      <c r="B64" s="5"/>
     </row>
     <row r="65" spans="1:2" ht="28.2" thickBot="1">
-      <c r="A65" s="3" t="s">
+      <c r="A65" s="6" t="s">
         <v>70</v>
       </c>
-      <c r="B65" s="3" t="s">
+      <c r="B65" s="6" t="s">
         <v>104</v>
       </c>
     </row>
     <row r="66" spans="1:2" ht="29.4" thickBot="1">
-      <c r="A66" s="5" t="s">
+      <c r="A66" s="4" t="s">
         <v>69</v>
       </c>
-      <c r="B66" s="6" t="s">
+      <c r="B66" s="5" t="s">
         <v>77</v>
       </c>
     </row>
     <row r="67" spans="1:2" ht="15" thickBot="1">
-      <c r="A67" s="5"/>
-      <c r="B67" s="6"/>
+      <c r="A67" s="4"/>
+      <c r="B67" s="5"/>
     </row>
     <row r="68" spans="1:2" ht="15" thickBot="1">
-      <c r="A68" s="3" t="s">
+      <c r="A68" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="B68" s="3" t="s">
+      <c r="B68" s="6" t="s">
         <v>79</v>
       </c>
     </row>
     <row r="69" spans="1:2" ht="15" thickBot="1">
-      <c r="A69" s="3" t="s">
+      <c r="A69" s="6" t="s">
+        <v>107</v>
+      </c>
+      <c r="B69" s="6" t="s">
         <v>108</v>
       </c>
-      <c r="B69" s="3" t="s">
-        <v>109</v>
-      </c>
     </row>
     <row r="70" spans="1:2" ht="15" thickBot="1">
-      <c r="A70" s="5"/>
-      <c r="B70" s="6"/>
+      <c r="A70" s="4"/>
+      <c r="B70" s="5"/>
     </row>
     <row r="71" spans="1:2" ht="15" thickBot="1">
-      <c r="A71" s="3" t="s">
+      <c r="A71" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="B71" s="3" t="s">
+      <c r="B71" s="6" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="72" spans="1:2" ht="28.8" thickBot="1">
-      <c r="A72" s="3" t="s">
-        <v>116</v>
-      </c>
-      <c r="B72" s="3" t="s">
-        <v>117</v>
+      <c r="A72" s="6" t="s">
+        <v>113</v>
+      </c>
+      <c r="B72" s="6" t="s">
+        <v>445</v>
       </c>
     </row>
     <row r="73" spans="1:2" ht="15" thickBot="1">
-      <c r="A73" s="5"/>
-      <c r="B73" s="6"/>
+      <c r="A73" s="4"/>
+      <c r="B73" s="5"/>
     </row>
     <row r="74" spans="1:2" ht="28.2" thickBot="1">
-      <c r="A74" s="3" t="s">
+      <c r="A74" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="B74" s="3" t="s">
+      <c r="B74" s="6" t="s">
         <v>84</v>
       </c>
     </row>
     <row r="75" spans="1:2" ht="15" thickBot="1">
-      <c r="A75" s="5"/>
-      <c r="B75" s="6"/>
+      <c r="A75" s="4"/>
+      <c r="B75" s="5"/>
     </row>
     <row r="76" spans="1:2" ht="15" thickBot="1">
-      <c r="A76" s="3" t="s">
+      <c r="A76" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="B76" s="3" t="s">
+      <c r="B76" s="6" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="77" spans="1:2" ht="15" thickBot="1">
-      <c r="A77" s="3" t="s">
-        <v>118</v>
-      </c>
-      <c r="B77" s="3" t="s">
-        <v>119</v>
+      <c r="A77" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="B77" s="6" t="s">
+        <v>446</v>
       </c>
     </row>
     <row r="78" spans="1:2" ht="15" thickBot="1">
-      <c r="A78" s="5"/>
-      <c r="B78" s="6"/>
+      <c r="A78" s="4"/>
+      <c r="B78" s="5"/>
     </row>
     <row r="79" spans="1:2" ht="28.2" thickBot="1">
-      <c r="A79" s="3" t="s">
+      <c r="A79" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B79" s="3" t="s">
+      <c r="B79" s="6" t="s">
         <v>85</v>
       </c>
     </row>
     <row r="80" spans="1:2" ht="15" thickBot="1">
-      <c r="A80" s="5"/>
-      <c r="B80" s="6"/>
+      <c r="A80" s="4"/>
+      <c r="B80" s="5"/>
     </row>
     <row r="81" spans="1:2" ht="15" thickBot="1">
-      <c r="A81" s="3" t="s">
+      <c r="A81" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="B81" s="3" t="s">
+      <c r="B81" s="6" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="82" spans="1:2" ht="15" thickBot="1">
-      <c r="A82" s="5"/>
-      <c r="B82" s="6"/>
+      <c r="A82" s="4"/>
+      <c r="B82" s="5"/>
     </row>
     <row r="83" spans="1:2" ht="28.2" thickBot="1">
-      <c r="A83" s="3" t="s">
+      <c r="A83" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="B83" s="3" t="s">
+      <c r="B83" s="6" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="84" spans="1:2" ht="15" thickBot="1">
-      <c r="A84" s="5"/>
-      <c r="B84" s="6"/>
+      <c r="A84" s="4"/>
+      <c r="B84" s="5"/>
     </row>
     <row r="85" spans="1:2" ht="28.2" thickBot="1">
-      <c r="A85" s="3" t="s">
+      <c r="A85" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="B85" s="3" t="s">
+      <c r="B85" s="6" t="s">
         <v>89</v>
       </c>
     </row>
     <row r="86" spans="1:2" ht="15" thickBot="1">
-      <c r="A86" s="5"/>
-      <c r="B86" s="6"/>
+      <c r="A86" s="4"/>
+      <c r="B86" s="5"/>
     </row>
     <row r="87" spans="1:2" ht="28.2" thickBot="1">
-      <c r="A87" s="3" t="s">
+      <c r="A87" s="6" t="s">
         <v>81</v>
       </c>
-      <c r="B87" s="3" t="s">
+      <c r="B87" s="6" t="s">
         <v>82</v>
       </c>
     </row>
     <row r="88" spans="1:2" ht="15" thickBot="1">
-      <c r="A88" s="5"/>
-      <c r="B88" s="6"/>
+      <c r="A88" s="4"/>
+      <c r="B88" s="5"/>
     </row>
     <row r="89" spans="1:2" ht="28.2" thickBot="1">
-      <c r="A89" s="3" t="s">
+      <c r="A89" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="B89" s="3" t="s">
+      <c r="B89" s="6" t="s">
         <v>90</v>
       </c>
     </row>
     <row r="90" spans="1:2" ht="15" thickBot="1">
-      <c r="A90" s="5"/>
-      <c r="B90" s="6"/>
+      <c r="A90" s="4"/>
+      <c r="B90" s="5"/>
     </row>
     <row r="91" spans="1:2" ht="28.2" thickBot="1">
-      <c r="A91" s="3" t="s">
+      <c r="A91" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="B91" s="3" t="s">
+      <c r="B91" s="6" t="s">
         <v>91</v>
       </c>
     </row>
     <row r="92" spans="1:2" ht="15" thickBot="1">
-      <c r="A92" s="5"/>
-      <c r="B92" s="6"/>
+      <c r="A92" s="4"/>
+      <c r="B92" s="5"/>
     </row>
     <row r="93" spans="1:2" ht="15" thickBot="1">
-      <c r="A93" s="3" t="s">
+      <c r="A93" s="6" t="s">
         <v>92</v>
       </c>
-      <c r="B93" s="3" t="s">
+      <c r="B93" s="6" t="s">
         <v>93</v>
       </c>
     </row>
     <row r="94" spans="1:2" ht="15" thickBot="1">
-      <c r="A94" s="5"/>
-      <c r="B94" s="6"/>
+      <c r="A94" s="4"/>
+      <c r="B94" s="5"/>
     </row>
     <row r="95" spans="1:2" ht="28.2" thickBot="1">
-      <c r="A95" s="3" t="s">
+      <c r="A95" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="B95" s="3" t="s">
+      <c r="B95" s="6" t="s">
         <v>86</v>
       </c>
     </row>
     <row r="96" spans="1:2" ht="15" thickBot="1">
-      <c r="A96" s="5"/>
-      <c r="B96" s="6"/>
+      <c r="A96" s="4"/>
+      <c r="B96" s="5"/>
     </row>
     <row r="97" spans="1:2" ht="15" thickBot="1">
-      <c r="A97" s="3" t="s">
+      <c r="A97" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="B97" s="3" t="s">
+      <c r="B97" s="6" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="98" spans="1:2" ht="15" thickBot="1">
-      <c r="A98" s="5"/>
-      <c r="B98" s="6"/>
+      <c r="A98" s="4"/>
+      <c r="B98" s="5"/>
     </row>
     <row r="99" spans="1:2" ht="28.2" thickBot="1">
-      <c r="A99" s="3" t="s">
+      <c r="A99" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="B99" s="3" t="s">
+      <c r="B99" s="6" t="s">
         <v>73</v>
       </c>
     </row>
     <row r="100" spans="1:2" ht="15" thickBot="1">
-      <c r="A100" s="5"/>
-      <c r="B100" s="6"/>
+      <c r="A100" s="4"/>
+      <c r="B100" s="5"/>
     </row>
     <row r="101" spans="1:2" ht="15" thickBot="1">
-      <c r="A101" s="3" t="s">
+      <c r="A101" s="6" t="s">
         <v>59</v>
       </c>
-      <c r="B101" s="3" t="s">
+      <c r="B101" s="6" t="s">
         <v>60</v>
       </c>
     </row>
     <row r="102" spans="1:2" ht="15" thickBot="1">
-      <c r="A102" s="5"/>
-      <c r="B102" s="6"/>
+      <c r="A102" s="4"/>
+      <c r="B102" s="5"/>
     </row>
     <row r="103" spans="1:2" ht="15" thickBot="1">
-      <c r="A103" s="3" t="s">
+      <c r="A103" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="B103" s="3" t="s">
+      <c r="B103" s="6" t="s">
         <v>105</v>
       </c>
     </row>
     <row r="104" spans="1:2" ht="15" thickBot="1">
-      <c r="A104" s="5"/>
-      <c r="B104" s="6"/>
+      <c r="A104" s="4"/>
+      <c r="B104" s="5"/>
     </row>
     <row r="105" spans="1:2" ht="28.2" thickBot="1">
-      <c r="A105" s="3" t="s">
+      <c r="A105" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="B105" s="3" t="s">
+      <c r="B105" s="6" t="s">
         <v>87</v>
       </c>
     </row>
     <row r="106" spans="1:2" ht="15" thickBot="1">
-      <c r="A106" s="5"/>
-      <c r="B106" s="6"/>
+      <c r="A106" s="4"/>
+      <c r="B106" s="5"/>
     </row>
     <row r="107" spans="1:2" ht="28.2" thickBot="1">
-      <c r="A107" s="3" t="s">
+      <c r="A107" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="B107" s="3" t="s">
+      <c r="B107" s="6" t="s">
         <v>88</v>
       </c>
     </row>
     <row r="108" spans="1:2" ht="28.2" thickBot="1">
-      <c r="A108" s="3" t="s">
-        <v>114</v>
-      </c>
-      <c r="B108" s="3" t="s">
-        <v>115</v>
+      <c r="A108" s="6" t="s">
+        <v>111</v>
+      </c>
+      <c r="B108" s="6" t="s">
+        <v>112</v>
       </c>
     </row>
     <row r="109" spans="1:2" ht="15" thickBot="1">
-      <c r="A109" s="5"/>
-      <c r="B109" s="6"/>
+      <c r="A109" s="4"/>
+      <c r="B109" s="5"/>
     </row>
     <row r="110" spans="1:2" ht="28.2" thickBot="1">
-      <c r="A110" s="3" t="s">
+      <c r="A110" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="B110" s="3" t="s">
+      <c r="B110" s="6" t="s">
         <v>94</v>
       </c>
     </row>
@@ -1592,4 +2839,1862 @@
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DCBFF228-6AD9-43F2-8D61-560CE4700E3A}">
+  <dimension ref="A1:B256"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
+  <cols>
+    <col min="1" max="1" width="40.33203125" style="8" customWidth="1"/>
+    <col min="2" max="2" width="37.77734375" style="8" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2">
+      <c r="A1" s="8" t="s">
+        <v>174</v>
+      </c>
+      <c r="B1" s="8" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2">
+      <c r="A2" s="8" t="s">
+        <v>116</v>
+      </c>
+      <c r="B2" s="8" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2">
+      <c r="A3" s="14" t="s">
+        <v>447</v>
+      </c>
+      <c r="B3" s="9" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2">
+      <c r="A4" s="14" t="s">
+        <v>448</v>
+      </c>
+      <c r="B4" s="9" t="s">
+        <v>449</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2">
+      <c r="A5" s="8" t="s">
+        <v>320</v>
+      </c>
+      <c r="B5" s="8" t="s">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2">
+      <c r="A6" s="8" t="s">
+        <v>334</v>
+      </c>
+      <c r="B6" s="8" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2">
+      <c r="A7" s="8" t="s">
+        <v>214</v>
+      </c>
+      <c r="B7" s="8" t="s">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2">
+      <c r="A8" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="B8" s="8" t="s">
+        <v>391</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2">
+      <c r="A9" s="14" t="s">
+        <v>29</v>
+      </c>
+      <c r="B9" s="9" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2">
+      <c r="A10" s="8" t="s">
+        <v>235</v>
+      </c>
+      <c r="B10" s="8" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2">
+      <c r="A11" s="8" t="s">
+        <v>281</v>
+      </c>
+      <c r="B11" s="8" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2">
+      <c r="A12" s="8" t="s">
+        <v>392</v>
+      </c>
+      <c r="B12" s="8" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2">
+      <c r="A13" s="8" t="s">
+        <v>176</v>
+      </c>
+      <c r="B13" s="8" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2">
+      <c r="A14" s="8" t="s">
+        <v>177</v>
+      </c>
+      <c r="B14" s="8" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2">
+      <c r="A15" s="14" t="s">
+        <v>450</v>
+      </c>
+      <c r="B15" s="9" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2">
+      <c r="A16" s="8" t="s">
+        <v>163</v>
+      </c>
+      <c r="B16" s="8" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2">
+      <c r="A17" s="8" t="s">
+        <v>147</v>
+      </c>
+      <c r="B17" s="8" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2">
+      <c r="A18" s="8" t="s">
+        <v>156</v>
+      </c>
+      <c r="B18" s="8" t="s">
+        <v>393</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2">
+      <c r="A19" s="8" t="s">
+        <v>287</v>
+      </c>
+      <c r="B19" s="8" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2">
+      <c r="A20" s="14" t="s">
+        <v>451</v>
+      </c>
+      <c r="B20" s="9" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2">
+      <c r="A21" s="8" t="s">
+        <v>297</v>
+      </c>
+      <c r="B21" s="8" t="s">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2">
+      <c r="A22" s="8" t="s">
+        <v>179</v>
+      </c>
+      <c r="B22" s="8" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2">
+      <c r="A23" s="8" t="s">
+        <v>285</v>
+      </c>
+      <c r="B23" s="8" t="s">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2">
+      <c r="A24" s="14" t="s">
+        <v>452</v>
+      </c>
+      <c r="B24" s="9" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2">
+      <c r="A25" s="8" t="s">
+        <v>318</v>
+      </c>
+      <c r="B25" s="8" t="s">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2">
+      <c r="A26" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="B26" s="9" t="s">
+        <v>453</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2">
+      <c r="A27" s="8" t="s">
+        <v>151</v>
+      </c>
+      <c r="B27" s="8" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2">
+      <c r="A28" s="8" t="s">
+        <v>352</v>
+      </c>
+      <c r="B28" s="8" t="s">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2">
+      <c r="A29" s="8" t="s">
+        <v>226</v>
+      </c>
+      <c r="B29" s="8" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2">
+      <c r="A30" s="8" t="s">
+        <v>149</v>
+      </c>
+      <c r="B30" s="8" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2">
+      <c r="A31" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="B31" s="8" t="s">
+        <v>454</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2">
+      <c r="A32" s="8" t="s">
+        <v>168</v>
+      </c>
+      <c r="B32" s="8" t="s">
+        <v>455</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2">
+      <c r="A33" s="8" t="s">
+        <v>145</v>
+      </c>
+      <c r="B33" s="8" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2">
+      <c r="A34" s="8" t="s">
+        <v>322</v>
+      </c>
+      <c r="B34" s="8" t="s">
+        <v>456</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2">
+      <c r="A35" s="8" t="s">
+        <v>227</v>
+      </c>
+      <c r="B35" s="8" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2">
+      <c r="A36" s="8" t="s">
+        <v>291</v>
+      </c>
+      <c r="B36" s="8" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2">
+      <c r="A37" s="8" t="s">
+        <v>396</v>
+      </c>
+      <c r="B37" s="8" t="s">
+        <v>395</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2">
+      <c r="A38" s="8" t="s">
+        <v>275</v>
+      </c>
+      <c r="B38" s="8" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2">
+      <c r="A39" s="8" t="s">
+        <v>397</v>
+      </c>
+      <c r="B39" s="8" t="s">
+        <v>398</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2">
+      <c r="A40" s="14" t="s">
+        <v>30</v>
+      </c>
+      <c r="B40" s="9" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2">
+      <c r="A41" s="14" t="s">
+        <v>458</v>
+      </c>
+      <c r="B41" s="9" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2">
+      <c r="A42" s="8" t="s">
+        <v>181</v>
+      </c>
+      <c r="B42" s="8" t="s">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2">
+      <c r="A43" s="8" t="s">
+        <v>293</v>
+      </c>
+      <c r="B43" s="8" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="44" spans="1:2">
+      <c r="A44" s="8" t="s">
+        <v>118</v>
+      </c>
+      <c r="B44" s="8" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="45" spans="1:2">
+      <c r="A45" s="14" t="s">
+        <v>459</v>
+      </c>
+      <c r="B45" s="9" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="46" spans="1:2">
+      <c r="A46" s="14" t="s">
+        <v>460</v>
+      </c>
+      <c r="B46" s="9" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="47" spans="1:2">
+      <c r="A47" s="8" t="s">
+        <v>374</v>
+      </c>
+      <c r="B47" s="8" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="48" spans="1:2">
+      <c r="A48" s="8" t="s">
+        <v>246</v>
+      </c>
+      <c r="B48" s="8" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="49" spans="1:2">
+      <c r="A49" s="8" t="s">
+        <v>248</v>
+      </c>
+      <c r="B49" s="8" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2">
+      <c r="A50" s="8" t="s">
+        <v>279</v>
+      </c>
+      <c r="B50" s="8" t="s">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="51" spans="1:2">
+      <c r="A51" s="8" t="s">
+        <v>461</v>
+      </c>
+      <c r="B51" s="8" t="s">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="52" spans="1:2">
+      <c r="A52" s="8" t="s">
+        <v>157</v>
+      </c>
+      <c r="B52" s="8" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="53" spans="1:2">
+      <c r="A53" s="14" t="s">
+        <v>462</v>
+      </c>
+      <c r="B53" s="9" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="54" spans="1:2">
+      <c r="A54" s="8" t="s">
+        <v>302</v>
+      </c>
+      <c r="B54" s="8" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="55" spans="1:2">
+      <c r="A55" s="8" t="s">
+        <v>306</v>
+      </c>
+      <c r="B55" s="8" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="56" spans="1:2">
+      <c r="A56" s="8" t="s">
+        <v>310</v>
+      </c>
+      <c r="B56" s="8" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="57" spans="1:2">
+      <c r="A57" s="8" t="s">
+        <v>161</v>
+      </c>
+      <c r="B57" s="8" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="58" spans="1:2">
+      <c r="A58" s="8" t="s">
+        <v>304</v>
+      </c>
+      <c r="B58" s="8" t="s">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="59" spans="1:2">
+      <c r="A59" s="8" t="s">
+        <v>308</v>
+      </c>
+      <c r="B59" s="8" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="60" spans="1:2">
+      <c r="A60" s="8" t="s">
+        <v>355</v>
+      </c>
+      <c r="B60" s="8" t="s">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="61" spans="1:2">
+      <c r="A61" s="8" t="s">
+        <v>426</v>
+      </c>
+      <c r="B61" s="8" t="s">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="62" spans="1:2">
+      <c r="A62" s="8" t="s">
+        <v>428</v>
+      </c>
+      <c r="B62" s="8" t="s">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="63" spans="1:2">
+      <c r="A63" s="8" t="s">
+        <v>429</v>
+      </c>
+      <c r="B63" s="8" t="s">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="64" spans="1:2">
+      <c r="A64" s="8" t="s">
+        <v>430</v>
+      </c>
+      <c r="B64" s="8" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="65" spans="1:2">
+      <c r="A65" s="8" t="s">
+        <v>120</v>
+      </c>
+      <c r="B65" s="8" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="66" spans="1:2">
+      <c r="A66" s="8" t="s">
+        <v>122</v>
+      </c>
+      <c r="B66" s="8" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="67" spans="1:2">
+      <c r="A67" s="8" t="s">
+        <v>233</v>
+      </c>
+      <c r="B67" s="8" t="s">
+        <v>399</v>
+      </c>
+    </row>
+    <row r="68" spans="1:2">
+      <c r="A68" s="8" t="s">
+        <v>411</v>
+      </c>
+      <c r="B68" s="8" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="69" spans="1:2">
+      <c r="A69" s="8" t="s">
+        <v>418</v>
+      </c>
+      <c r="B69" s="8" t="s">
+        <v>419</v>
+      </c>
+    </row>
+    <row r="70" spans="1:2">
+      <c r="A70" s="8" t="s">
+        <v>415</v>
+      </c>
+      <c r="B70" s="8" t="s">
+        <v>414</v>
+      </c>
+    </row>
+    <row r="71" spans="1:2">
+      <c r="A71" s="8" t="s">
+        <v>408</v>
+      </c>
+      <c r="B71" s="8" t="s">
+        <v>409</v>
+      </c>
+    </row>
+    <row r="72" spans="1:2">
+      <c r="A72" s="8" t="s">
+        <v>234</v>
+      </c>
+      <c r="B72" s="8" t="s">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="73" spans="1:2">
+      <c r="A73" s="8" t="s">
+        <v>124</v>
+      </c>
+      <c r="B73" s="8" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="74" spans="1:2">
+      <c r="A74" s="8" t="s">
+        <v>416</v>
+      </c>
+      <c r="B74" s="8" t="s">
+        <v>417</v>
+      </c>
+    </row>
+    <row r="75" spans="1:2">
+      <c r="A75" s="8" t="s">
+        <v>299</v>
+      </c>
+      <c r="B75" s="8" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="76" spans="1:2">
+      <c r="A76" s="8" t="s">
+        <v>412</v>
+      </c>
+      <c r="B76" s="8" t="s">
+        <v>413</v>
+      </c>
+    </row>
+    <row r="77" spans="1:2">
+      <c r="A77" s="8" t="s">
+        <v>406</v>
+      </c>
+      <c r="B77" s="8" t="s">
+        <v>407</v>
+      </c>
+    </row>
+    <row r="78" spans="1:2">
+      <c r="A78" s="8" t="s">
+        <v>231</v>
+      </c>
+      <c r="B78" s="8" t="s">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="79" spans="1:2">
+      <c r="A79" s="8" t="s">
+        <v>232</v>
+      </c>
+      <c r="B79" s="8" t="s">
+        <v>401</v>
+      </c>
+    </row>
+    <row r="80" spans="1:2">
+      <c r="A80" s="8" t="s">
+        <v>312</v>
+      </c>
+      <c r="B80" s="8" t="s">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="81" spans="1:2">
+      <c r="A81" s="8" t="s">
+        <v>420</v>
+      </c>
+      <c r="B81" s="8" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="82" spans="1:2">
+      <c r="A82" s="8" t="s">
+        <v>155</v>
+      </c>
+      <c r="B82" s="8" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="83" spans="1:2">
+      <c r="A83" s="8" t="s">
+        <v>362</v>
+      </c>
+      <c r="B83" s="8" t="s">
+        <v>363</v>
+      </c>
+    </row>
+    <row r="84" spans="1:2">
+      <c r="A84" s="8" t="s">
+        <v>169</v>
+      </c>
+      <c r="B84" s="8" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="85" spans="1:2">
+      <c r="A85" s="8" t="s">
+        <v>357</v>
+      </c>
+      <c r="B85" s="8" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="86" spans="1:2">
+      <c r="A86" s="8" t="s">
+        <v>165</v>
+      </c>
+      <c r="B86" s="8" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="87" spans="1:2">
+      <c r="A87" s="8" t="s">
+        <v>366</v>
+      </c>
+      <c r="B87" s="8" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="88" spans="1:2">
+      <c r="A88" s="8" t="s">
+        <v>171</v>
+      </c>
+      <c r="B88" s="8" t="s">
+        <v>423</v>
+      </c>
+    </row>
+    <row r="89" spans="1:2">
+      <c r="A89" s="8" t="s">
+        <v>141</v>
+      </c>
+      <c r="B89" s="8" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="90" spans="1:2">
+      <c r="A90" s="8" t="s">
+        <v>314</v>
+      </c>
+      <c r="B90" s="8" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="91" spans="1:2">
+      <c r="A91" s="8" t="s">
+        <v>316</v>
+      </c>
+      <c r="B91" s="8" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="92" spans="1:2">
+      <c r="A92" s="8" t="s">
+        <v>213</v>
+      </c>
+      <c r="B92" s="8" t="s">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="93" spans="1:2">
+      <c r="A93" s="8" t="s">
+        <v>359</v>
+      </c>
+      <c r="B93" s="8" t="s">
+        <v>437</v>
+      </c>
+    </row>
+    <row r="94" spans="1:2">
+      <c r="A94" s="8" t="s">
+        <v>167</v>
+      </c>
+      <c r="B94" s="8" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="95" spans="1:2">
+      <c r="A95" s="8" t="s">
+        <v>360</v>
+      </c>
+      <c r="B95" s="8" t="s">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="96" spans="1:2">
+      <c r="A96" s="8" t="s">
+        <v>239</v>
+      </c>
+      <c r="B96" s="8" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="97" spans="1:2">
+      <c r="A97" s="8" t="s">
+        <v>358</v>
+      </c>
+      <c r="B97" s="8" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="98" spans="1:2">
+      <c r="A98" s="8" t="s">
+        <v>439</v>
+      </c>
+      <c r="B98" s="8" t="s">
+        <v>440</v>
+      </c>
+    </row>
+    <row r="99" spans="1:2">
+      <c r="A99" s="8" t="s">
+        <v>364</v>
+      </c>
+      <c r="B99" s="8" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="100" spans="1:2">
+      <c r="A100" s="8" t="s">
+        <v>170</v>
+      </c>
+      <c r="B100" s="8" t="s">
+        <v>425</v>
+      </c>
+    </row>
+    <row r="101" spans="1:2">
+      <c r="A101" s="8" t="s">
+        <v>441</v>
+      </c>
+      <c r="B101" s="8" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="102" spans="1:2">
+      <c r="A102" s="8" t="s">
+        <v>182</v>
+      </c>
+      <c r="B102" s="8" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="103" spans="1:2">
+      <c r="A103" s="8" t="s">
+        <v>209</v>
+      </c>
+      <c r="B103" s="8" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="104" spans="1:2">
+      <c r="A104" s="8" t="s">
+        <v>344</v>
+      </c>
+      <c r="B104" s="8" t="s">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="105" spans="1:2">
+      <c r="A105" s="8" t="s">
+        <v>323</v>
+      </c>
+      <c r="B105" s="8" t="s">
+        <v>324</v>
+      </c>
+    </row>
+    <row r="106" spans="1:2">
+      <c r="A106" s="8" t="s">
+        <v>336</v>
+      </c>
+      <c r="B106" s="8" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="107" spans="1:2">
+      <c r="A107" s="8" t="s">
+        <v>211</v>
+      </c>
+      <c r="B107" s="8" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="108" spans="1:2">
+      <c r="A108" s="8" t="s">
+        <v>241</v>
+      </c>
+      <c r="B108" s="8" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="109" spans="1:2">
+      <c r="A109" s="8" t="s">
+        <v>245</v>
+      </c>
+      <c r="B109" s="8" t="s">
+        <v>463</v>
+      </c>
+    </row>
+    <row r="110" spans="1:2">
+      <c r="A110" s="8" t="s">
+        <v>250</v>
+      </c>
+      <c r="B110" s="8" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="111" spans="1:2">
+      <c r="A111" s="8" t="s">
+        <v>243</v>
+      </c>
+      <c r="B111" s="8" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="112" spans="1:2">
+      <c r="A112" s="8" t="s">
+        <v>338</v>
+      </c>
+      <c r="B112" s="8" t="s">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="113" spans="1:2">
+      <c r="A113" s="8" t="s">
+        <v>464</v>
+      </c>
+      <c r="B113" s="8" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="114" spans="1:2">
+      <c r="A114" s="8" t="s">
+        <v>466</v>
+      </c>
+      <c r="B114" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="115" spans="1:2">
+      <c r="A115" s="14" t="s">
+        <v>467</v>
+      </c>
+      <c r="B115" s="9" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="116" spans="1:2">
+      <c r="A116" s="8" t="s">
+        <v>367</v>
+      </c>
+      <c r="B116" s="8" t="s">
+        <v>368</v>
+      </c>
+    </row>
+    <row r="117" spans="1:2">
+      <c r="A117" s="8" t="s">
+        <v>184</v>
+      </c>
+      <c r="B117" s="12" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="118" spans="1:2">
+      <c r="A118" s="8" t="s">
+        <v>126</v>
+      </c>
+      <c r="B118" s="8" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="119" spans="1:2">
+      <c r="A119" s="8" t="s">
+        <v>128</v>
+      </c>
+      <c r="B119" s="8" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="120" spans="1:2">
+      <c r="A120" s="8" t="s">
+        <v>258</v>
+      </c>
+      <c r="B120" s="8" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="121" spans="1:2">
+      <c r="A121" s="8" t="s">
+        <v>256</v>
+      </c>
+      <c r="B121" s="8" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="122" spans="1:2">
+      <c r="A122" s="8" t="s">
+        <v>254</v>
+      </c>
+      <c r="B122" s="8" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="123" spans="1:2">
+      <c r="A123" s="8" t="s">
+        <v>260</v>
+      </c>
+      <c r="B123" s="8" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="124" spans="1:2">
+      <c r="A124" s="8" t="s">
+        <v>185</v>
+      </c>
+      <c r="B124" s="8" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="125" spans="1:2">
+      <c r="A125" s="8" t="s">
+        <v>237</v>
+      </c>
+      <c r="B125" s="8" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="126" spans="1:2">
+      <c r="A126" s="15" t="s">
+        <v>468</v>
+      </c>
+      <c r="B126" s="12" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="127" spans="1:2">
+      <c r="A127" s="8" t="s">
+        <v>130</v>
+      </c>
+      <c r="B127" s="8" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="128" spans="1:2">
+      <c r="A128" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="B128" s="8" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="129" spans="1:2">
+      <c r="A129" s="8" t="s">
+        <v>132</v>
+      </c>
+      <c r="B129" s="8" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="130" spans="1:2">
+      <c r="A130" s="15" t="s">
+        <v>469</v>
+      </c>
+      <c r="B130" s="12" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="131" spans="1:2">
+      <c r="A131" s="8" t="s">
+        <v>388</v>
+      </c>
+      <c r="B131" s="8" t="s">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="132" spans="1:2">
+      <c r="A132" s="15" t="s">
+        <v>470</v>
+      </c>
+      <c r="B132" s="12" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="133" spans="1:2">
+      <c r="A133" s="8" t="s">
+        <v>325</v>
+      </c>
+      <c r="B133" s="12" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="134" spans="1:2">
+      <c r="A134" s="8" t="s">
+        <v>187</v>
+      </c>
+      <c r="B134" s="8" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="135" spans="1:2">
+      <c r="A135" s="8" t="s">
+        <v>326</v>
+      </c>
+      <c r="B135" s="8" t="s">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="136" spans="1:2">
+      <c r="A136" s="8" t="s">
+        <v>472</v>
+      </c>
+      <c r="B136" t="s">
+        <v>471</v>
+      </c>
+    </row>
+    <row r="137" spans="1:2">
+      <c r="A137" s="8" t="s">
+        <v>134</v>
+      </c>
+      <c r="B137" s="8" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="138" spans="1:2">
+      <c r="A138" s="8" t="s">
+        <v>262</v>
+      </c>
+      <c r="B138" s="8" t="s">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="139" spans="1:2">
+      <c r="A139" s="8" t="s">
+        <v>346</v>
+      </c>
+      <c r="B139" s="8" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="140" spans="1:2">
+      <c r="A140" s="8" t="s">
+        <v>277</v>
+      </c>
+      <c r="B140" s="8" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="141" spans="1:2">
+      <c r="A141" s="8" t="s">
+        <v>328</v>
+      </c>
+      <c r="B141" s="8" t="s">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="142" spans="1:2">
+      <c r="A142" s="8" t="s">
+        <v>136</v>
+      </c>
+      <c r="B142" s="8" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="143" spans="1:2">
+      <c r="A143" s="8" t="s">
+        <v>382</v>
+      </c>
+      <c r="B143" s="8" t="s">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="144" spans="1:2">
+      <c r="A144" s="8" t="s">
+        <v>283</v>
+      </c>
+      <c r="B144" s="8" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="145" spans="1:2">
+      <c r="A145" s="15" t="s">
+        <v>473</v>
+      </c>
+      <c r="B145" s="12" t="s">
+        <v>474</v>
+      </c>
+    </row>
+    <row r="146" spans="1:2">
+      <c r="A146" s="8" t="s">
+        <v>340</v>
+      </c>
+      <c r="B146" s="8" t="s">
+        <v>341</v>
+      </c>
+    </row>
+    <row r="147" spans="1:2">
+      <c r="A147" s="8" t="s">
+        <v>330</v>
+      </c>
+      <c r="B147" s="8" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="148" spans="1:2">
+      <c r="A148" s="8" t="s">
+        <v>137</v>
+      </c>
+      <c r="B148" s="8" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="149" spans="1:2">
+      <c r="A149" s="8" t="s">
+        <v>153</v>
+      </c>
+      <c r="B149" s="8" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="150" spans="1:2">
+      <c r="A150" s="15" t="s">
+        <v>475</v>
+      </c>
+      <c r="B150" s="12" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="151" spans="1:2">
+      <c r="A151" s="8" t="s">
+        <v>139</v>
+      </c>
+      <c r="B151" s="8" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="152" spans="1:2">
+      <c r="A152" s="8" t="s">
+        <v>189</v>
+      </c>
+      <c r="B152" s="8" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="153" spans="1:2">
+      <c r="A153" s="15" t="s">
+        <v>476</v>
+      </c>
+      <c r="B153" s="12" t="s">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="154" spans="1:2">
+      <c r="A154" s="8" t="s">
+        <v>191</v>
+      </c>
+      <c r="B154" s="8" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="155" spans="1:2">
+      <c r="A155" s="8" t="s">
+        <v>193</v>
+      </c>
+      <c r="B155" s="8" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="156" spans="1:2">
+      <c r="A156" s="8" t="s">
+        <v>159</v>
+      </c>
+      <c r="B156" s="8" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="157" spans="1:2">
+      <c r="A157" s="8" t="s">
+        <v>271</v>
+      </c>
+      <c r="B157" s="8" t="s">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="158" spans="1:2">
+      <c r="A158" s="8" t="s">
+        <v>269</v>
+      </c>
+      <c r="B158" s="8" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="159" spans="1:2">
+      <c r="A159" s="8" t="s">
+        <v>273</v>
+      </c>
+      <c r="B159" s="8" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="160" spans="1:2">
+      <c r="A160" s="8" t="s">
+        <v>265</v>
+      </c>
+      <c r="B160" s="8" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="161" spans="1:2">
+      <c r="A161" s="8" t="s">
+        <v>267</v>
+      </c>
+      <c r="B161" s="8" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="162" spans="1:2">
+      <c r="A162" s="8" t="s">
+        <v>252</v>
+      </c>
+      <c r="B162" s="8" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="163" spans="1:2">
+      <c r="A163" s="8" t="s">
+        <v>263</v>
+      </c>
+      <c r="B163" s="8" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="164" spans="1:2">
+      <c r="A164" s="8" t="s">
+        <v>195</v>
+      </c>
+      <c r="B164" s="8" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="165" spans="1:2">
+      <c r="A165" s="15" t="s">
+        <v>477</v>
+      </c>
+      <c r="B165" s="12" t="s">
+        <v>478</v>
+      </c>
+    </row>
+    <row r="166" spans="1:2">
+      <c r="A166" s="15" t="s">
+        <v>25</v>
+      </c>
+      <c r="B166" s="12" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="167" spans="1:2">
+      <c r="A167" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="B167" s="12" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="168" spans="1:2">
+      <c r="A168" s="8" t="s">
+        <v>197</v>
+      </c>
+      <c r="B168" s="8" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="169" spans="1:2">
+      <c r="A169" s="8" t="s">
+        <v>369</v>
+      </c>
+      <c r="B169" s="8" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="170" spans="1:2">
+      <c r="A170" s="8" t="s">
+        <v>203</v>
+      </c>
+      <c r="B170" s="8" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="171" spans="1:2">
+      <c r="A171" s="8" t="s">
+        <v>342</v>
+      </c>
+      <c r="B171" s="8" t="s">
+        <v>343</v>
+      </c>
+    </row>
+    <row r="172" spans="1:2">
+      <c r="A172" s="8" t="s">
+        <v>229</v>
+      </c>
+      <c r="B172" s="8" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="173" spans="1:2">
+      <c r="A173" s="8" t="s">
+        <v>220</v>
+      </c>
+      <c r="B173" s="8" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="174" spans="1:2">
+      <c r="A174" s="8" t="s">
+        <v>172</v>
+      </c>
+      <c r="B174" s="8" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="175" spans="1:2">
+      <c r="A175" s="8" t="s">
+        <v>143</v>
+      </c>
+      <c r="B175" s="8" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="176" spans="1:2">
+      <c r="A176" s="8" t="s">
+        <v>386</v>
+      </c>
+      <c r="B176" s="8" t="s">
+        <v>387</v>
+      </c>
+    </row>
+    <row r="177" spans="1:2">
+      <c r="A177" s="8" t="s">
+        <v>289</v>
+      </c>
+      <c r="B177" s="8" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="178" spans="1:2">
+      <c r="A178" s="15" t="s">
+        <v>479</v>
+      </c>
+      <c r="B178" s="12" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="179" spans="1:2">
+      <c r="A179" s="15" t="s">
+        <v>480</v>
+      </c>
+      <c r="B179" s="12" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="180" spans="1:2">
+      <c r="A180" s="15" t="s">
+        <v>481</v>
+      </c>
+      <c r="B180" s="12" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="181" spans="1:2">
+      <c r="A181" s="8" t="s">
+        <v>295</v>
+      </c>
+      <c r="B181" s="8" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="182" spans="1:2">
+      <c r="A182" s="8" t="s">
+        <v>224</v>
+      </c>
+      <c r="B182" s="8" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="183" spans="1:2">
+      <c r="A183" s="8" t="s">
+        <v>215</v>
+      </c>
+      <c r="B183" s="8" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="184" spans="1:2">
+      <c r="A184" s="8" t="s">
+        <v>207</v>
+      </c>
+      <c r="B184" t="s">
+        <v>483</v>
+      </c>
+    </row>
+    <row r="185" spans="1:2">
+      <c r="A185" s="8" t="s">
+        <v>380</v>
+      </c>
+      <c r="B185" s="8" t="s">
+        <v>381</v>
+      </c>
+    </row>
+    <row r="186" spans="1:2">
+      <c r="A186" s="8" t="s">
+        <v>378</v>
+      </c>
+      <c r="B186" s="8" t="s">
+        <v>379</v>
+      </c>
+    </row>
+    <row r="187" spans="1:2">
+      <c r="A187" s="8" t="s">
+        <v>376</v>
+      </c>
+      <c r="B187" s="8" t="s">
+        <v>377</v>
+      </c>
+    </row>
+    <row r="188" spans="1:2">
+      <c r="A188" s="15" t="s">
+        <v>482</v>
+      </c>
+      <c r="B188" s="12" t="s">
+        <v>484</v>
+      </c>
+    </row>
+    <row r="189" spans="1:2">
+      <c r="A189" s="8" t="s">
+        <v>205</v>
+      </c>
+      <c r="B189" s="8" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="190" spans="1:2">
+      <c r="A190" s="8" t="s">
+        <v>348</v>
+      </c>
+      <c r="B190" s="8" t="s">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="191" spans="1:2">
+      <c r="A191" s="15" t="s">
+        <v>485</v>
+      </c>
+      <c r="B191" s="12" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="192" spans="1:2">
+      <c r="A192" s="15" t="s">
+        <v>486</v>
+      </c>
+      <c r="B192" s="12" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="193" spans="1:2">
+      <c r="A193" s="8" t="s">
+        <v>199</v>
+      </c>
+      <c r="B193" s="8" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="194" spans="1:2">
+      <c r="A194" s="8" t="s">
+        <v>384</v>
+      </c>
+      <c r="B194" s="8" t="s">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="195" spans="1:2">
+      <c r="A195" s="15" t="s">
+        <v>487</v>
+      </c>
+      <c r="B195" s="12" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="196" spans="1:2">
+      <c r="A196" s="15" t="s">
+        <v>488</v>
+      </c>
+      <c r="B196" s="12" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="197" spans="1:2">
+      <c r="A197" s="17" t="s">
+        <v>222</v>
+      </c>
+      <c r="B197" s="17" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="198" spans="1:2" ht="15" thickBot="1">
+      <c r="A198" s="17" t="s">
+        <v>201</v>
+      </c>
+      <c r="B198" s="17" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="199" spans="1:2" ht="15" thickBot="1">
+      <c r="A199" s="13" t="s">
+        <v>219</v>
+      </c>
+      <c r="B199" s="13" t="s">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="200" spans="1:2" ht="15" thickBot="1">
+      <c r="A200" s="16" t="s">
+        <v>489</v>
+      </c>
+      <c r="B200" s="11" t="s">
+        <v>490</v>
+      </c>
+    </row>
+    <row r="201" spans="1:2" ht="15" thickBot="1">
+      <c r="A201" s="13" t="s">
+        <v>217</v>
+      </c>
+      <c r="B201" s="13" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="202" spans="1:2" ht="15" thickBot="1">
+      <c r="A202" s="16" t="s">
+        <v>13</v>
+      </c>
+      <c r="B202" s="11" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="203" spans="1:2" ht="15" thickBot="1">
+      <c r="A203" s="13" t="s">
+        <v>332</v>
+      </c>
+      <c r="B203" s="13" t="s">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="204" spans="1:2" ht="15" thickBot="1">
+      <c r="A204" s="16" t="s">
+        <v>12</v>
+      </c>
+      <c r="B204" s="11" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="205" spans="1:2" ht="15" thickBot="1">
+      <c r="A205" s="16"/>
+      <c r="B205" s="11"/>
+    </row>
+    <row r="206" spans="1:2" ht="15" thickBot="1">
+      <c r="A206" s="16"/>
+      <c r="B206" s="11"/>
+    </row>
+    <row r="207" spans="1:2" ht="15" thickBot="1">
+      <c r="A207" s="13"/>
+      <c r="B207" s="13"/>
+    </row>
+    <row r="208" spans="1:2" ht="15" thickBot="1">
+      <c r="A208" s="4"/>
+      <c r="B208" s="10"/>
+    </row>
+    <row r="209" spans="1:2" ht="15" thickBot="1">
+      <c r="A209" s="4"/>
+      <c r="B209" s="10"/>
+    </row>
+    <row r="210" spans="1:2" ht="15" thickBot="1">
+      <c r="A210" s="4"/>
+      <c r="B210" s="10"/>
+    </row>
+    <row r="211" spans="1:2" ht="15" thickBot="1">
+      <c r="A211" s="4"/>
+      <c r="B211" s="10"/>
+    </row>
+    <row r="212" spans="1:2" ht="15" thickBot="1">
+      <c r="A212" s="4"/>
+      <c r="B212" s="10"/>
+    </row>
+    <row r="213" spans="1:2" ht="15" thickBot="1">
+      <c r="A213" s="4"/>
+      <c r="B213" s="10"/>
+    </row>
+    <row r="214" spans="1:2" ht="15" thickBot="1">
+      <c r="A214" s="4"/>
+      <c r="B214" s="10"/>
+    </row>
+    <row r="215" spans="1:2" ht="15" thickBot="1">
+      <c r="A215" s="4"/>
+      <c r="B215" s="10"/>
+    </row>
+    <row r="216" spans="1:2" ht="15" thickBot="1">
+      <c r="A216" s="4"/>
+      <c r="B216" s="10"/>
+    </row>
+    <row r="217" spans="1:2" ht="15" thickBot="1">
+      <c r="A217" s="4"/>
+      <c r="B217" s="10"/>
+    </row>
+    <row r="218" spans="1:2" ht="15" thickBot="1">
+      <c r="A218" s="4"/>
+      <c r="B218" s="10"/>
+    </row>
+    <row r="219" spans="1:2" ht="15" thickBot="1">
+      <c r="A219" s="4"/>
+      <c r="B219" s="10"/>
+    </row>
+    <row r="220" spans="1:2" ht="15" thickBot="1">
+      <c r="A220" s="4"/>
+      <c r="B220" s="10"/>
+    </row>
+    <row r="221" spans="1:2" ht="15" thickBot="1">
+      <c r="A221" s="4"/>
+      <c r="B221" s="10"/>
+    </row>
+    <row r="222" spans="1:2" ht="15" thickBot="1">
+      <c r="A222" s="4"/>
+      <c r="B222" s="10"/>
+    </row>
+    <row r="223" spans="1:2" ht="15" thickBot="1">
+      <c r="A223" s="4"/>
+      <c r="B223" s="10"/>
+    </row>
+    <row r="224" spans="1:2" ht="15" thickBot="1">
+      <c r="A224" s="4"/>
+      <c r="B224" s="10"/>
+    </row>
+    <row r="225" spans="1:2" ht="15" thickBot="1">
+      <c r="A225" s="4"/>
+      <c r="B225" s="10"/>
+    </row>
+    <row r="226" spans="1:2" ht="15" thickBot="1">
+      <c r="A226" s="4"/>
+      <c r="B226" s="10"/>
+    </row>
+    <row r="227" spans="1:2" ht="15" thickBot="1">
+      <c r="A227" s="4"/>
+      <c r="B227" s="10"/>
+    </row>
+    <row r="228" spans="1:2" ht="15" thickBot="1">
+      <c r="A228" s="4"/>
+      <c r="B228" s="10"/>
+    </row>
+    <row r="229" spans="1:2" ht="15" thickBot="1">
+      <c r="A229" s="4"/>
+      <c r="B229" s="10"/>
+    </row>
+    <row r="230" spans="1:2" ht="15" thickBot="1">
+      <c r="A230" s="4"/>
+      <c r="B230" s="10"/>
+    </row>
+    <row r="231" spans="1:2" ht="15" thickBot="1">
+      <c r="A231" s="4"/>
+      <c r="B231" s="10"/>
+    </row>
+    <row r="232" spans="1:2" ht="15" thickBot="1">
+      <c r="A232" s="4"/>
+      <c r="B232" s="10"/>
+    </row>
+    <row r="233" spans="1:2" ht="15" thickBot="1">
+      <c r="A233" s="4"/>
+      <c r="B233" s="10"/>
+    </row>
+    <row r="234" spans="1:2" ht="15" thickBot="1">
+      <c r="A234" s="4"/>
+      <c r="B234" s="10"/>
+    </row>
+    <row r="235" spans="1:2" ht="15" thickBot="1">
+      <c r="A235" s="4"/>
+      <c r="B235" s="10"/>
+    </row>
+    <row r="236" spans="1:2" ht="15" thickBot="1">
+      <c r="A236" s="4"/>
+      <c r="B236" s="10"/>
+    </row>
+    <row r="237" spans="1:2" ht="15" thickBot="1">
+      <c r="A237" s="4"/>
+      <c r="B237" s="10"/>
+    </row>
+    <row r="238" spans="1:2" ht="15" thickBot="1">
+      <c r="A238" s="4"/>
+      <c r="B238" s="10"/>
+    </row>
+    <row r="239" spans="1:2" ht="15" thickBot="1">
+      <c r="A239" s="4"/>
+      <c r="B239" s="10"/>
+    </row>
+    <row r="240" spans="1:2" ht="15" thickBot="1">
+      <c r="A240" s="4"/>
+      <c r="B240" s="10"/>
+    </row>
+    <row r="241" spans="1:2" ht="15" thickBot="1">
+      <c r="A241" s="4"/>
+      <c r="B241" s="10"/>
+    </row>
+    <row r="242" spans="1:2" ht="15" thickBot="1">
+      <c r="A242" s="4"/>
+      <c r="B242" s="10"/>
+    </row>
+    <row r="243" spans="1:2" ht="15" thickBot="1">
+      <c r="A243" s="4"/>
+      <c r="B243" s="10"/>
+    </row>
+    <row r="244" spans="1:2" ht="15" thickBot="1">
+      <c r="A244" s="4"/>
+      <c r="B244" s="10"/>
+    </row>
+    <row r="245" spans="1:2" ht="15" thickBot="1">
+      <c r="A245" s="4"/>
+      <c r="B245" s="10"/>
+    </row>
+    <row r="246" spans="1:2" ht="15" thickBot="1">
+      <c r="A246" s="4"/>
+      <c r="B246" s="10"/>
+    </row>
+    <row r="247" spans="1:2" ht="15" thickBot="1">
+      <c r="A247" s="4"/>
+      <c r="B247" s="10"/>
+    </row>
+    <row r="248" spans="1:2" ht="15" thickBot="1">
+      <c r="A248" s="4"/>
+      <c r="B248" s="10"/>
+    </row>
+    <row r="249" spans="1:2" ht="15" thickBot="1">
+      <c r="A249" s="4"/>
+      <c r="B249" s="10"/>
+    </row>
+    <row r="250" spans="1:2" ht="15" thickBot="1">
+      <c r="A250" s="4"/>
+      <c r="B250" s="10"/>
+    </row>
+    <row r="251" spans="1:2" ht="15" thickBot="1">
+      <c r="A251" s="4"/>
+      <c r="B251" s="10"/>
+    </row>
+    <row r="252" spans="1:2" ht="15" thickBot="1">
+      <c r="A252" s="4"/>
+      <c r="B252" s="10"/>
+    </row>
+    <row r="253" spans="1:2" ht="15" thickBot="1">
+      <c r="A253" s="4"/>
+      <c r="B253" s="10"/>
+    </row>
+    <row r="254" spans="1:2" ht="15" thickBot="1">
+      <c r="A254" s="4"/>
+      <c r="B254" s="10"/>
+    </row>
+    <row r="255" spans="1:2" ht="15" thickBot="1">
+      <c r="A255" s="4"/>
+      <c r="B255" s="10"/>
+    </row>
+    <row r="256" spans="1:2" ht="15" thickBot="1">
+      <c r="A256" s="4"/>
+      <c r="B256" s="10"/>
+    </row>
+  </sheetData>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A1:B257">
+    <sortCondition ref="A211:A257"/>
+  </sortState>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Adjusted content regarding styling, validating, external components, website integration to version 2.0.0
</commit_message>
<xml_diff>
--- a/docu-content/010_Documentation/200_Terminology/SortedList_of_Terms.xlsx
+++ b/docu-content/010_Documentation/200_Terminology/SortedList_of_Terms.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aklep\WebstormProjects\Freon-documentation\docu-content\010_Documentation\200_Terminology\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{51154000-4CF9-4945-B87D-6262E1C33001}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05D2ED58-81E3-4FF6-BDA5-8223453F0BEE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" activeTab="1" xr2:uid="{DB8CC088-8583-4FF2-9A6E-2F9270EA0E65}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="528" uniqueCount="491">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="524" uniqueCount="495">
   <si>
     <t>named property projection</t>
   </si>
@@ -397,9 +397,6 @@
     <t>Freon</t>
   </si>
   <si>
-    <t>The Freon framework for building DSL editors for the web; also the Frisian word for “friend.”</t>
-  </si>
-  <si>
     <t>Freon interpreter framework</t>
   </si>
   <si>
@@ -415,12 +412,6 @@
     <t>LionWeb repository</t>
   </si>
   <si>
-    <t>A server implementation that stores models using the LionWeb protocol; can be connected to Freon for model persistence.</t>
-  </si>
-  <si>
-    <t>Model unit</t>
-  </si>
-  <si>
     <t>A modular part of a model that can be edited or stored separately, enabling large-scale DSL models.</t>
   </si>
   <si>
@@ -445,9 +436,6 @@
     <t>The visual representation of the model’s AST displayed and manipulated in the Freon editor.</t>
   </si>
   <si>
-    <t>Projectional editing</t>
-  </si>
-  <si>
     <t>An editing paradigm where users work directly on the model structure (AST) instead of plain text.</t>
   </si>
   <si>
@@ -520,9 +508,6 @@
     <t>Box API</t>
   </si>
   <si>
-    <t>Key editor box methods such as findParam(), setFocus(), and refreshComponent().</t>
-  </si>
-  <si>
     <t>FreScoper Interface</t>
   </si>
   <si>
@@ -580,9 +565,6 @@
     <t>A concept representing a grading rule composed of a grade and an expression.</t>
   </si>
   <si>
-    <t>Limited concept</t>
-  </si>
-  <si>
     <t>Metamodel</t>
   </si>
   <si>
@@ -595,9 +577,6 @@
     <t>A rule allowing one namespace to import names from another (e.g., from a related page).</t>
   </si>
   <si>
-    <t>Projectional editor</t>
-  </si>
-  <si>
     <t>An editor that directly manipulates the AST, ensuring models are always syntactically valid.</t>
   </si>
   <si>
@@ -643,12 +622,6 @@
     <t>The three main components of Freon’s semantic analysis framework.</t>
   </si>
   <si>
-    <t>Type Provider (Typer)</t>
-  </si>
-  <si>
-    <t>A definition (.type) file that specifies typing rules for a language.</t>
-  </si>
-  <si>
     <t>Type Concept</t>
   </si>
   <si>
@@ -667,6 +640,9 @@
     <t>Defines how to determine the type of a term, e.g. infertype self.declaredType.</t>
   </si>
   <si>
+    <t>Limited Concept</t>
+  </si>
+  <si>
     <t>FreType Interface</t>
   </si>
   <si>
@@ -889,12 +865,12 @@
     <t>A tree representing how a model appears visually; in Freon, this corresponds to the Box Model.</t>
   </si>
   <si>
-    <t>Box Tree</t>
-  </si>
-  <si>
     <t>The hierarchy of boxes used by the Freon editor to represent layout and structure of a model on screen.</t>
   </si>
   <si>
+    <t>Projectional Editing</t>
+  </si>
+  <si>
     <t>Svelte Components</t>
   </si>
   <si>
@@ -1021,9 +997,6 @@
     <t>Private Properties</t>
   </si>
   <si>
-    <t>Properties in .ast files marked with the private keyword; visible only within their own namespace, not when imported elsewhere.</t>
-  </si>
-  <si>
     <t>Visible Nodes</t>
   </si>
   <si>
@@ -1210,47 +1183,6 @@
     <t>An identifier assigned to a box that links it to specific editor behaviors or actions. Box roles connect visual elements in a projection to the logic that handles user interactions.</t>
   </si>
   <si>
-    <r>
-      <t>Definition of user-defined error messages and severity levels (</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Arial Unicode MS"/>
-      </rPr>
-      <t>message</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">, </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Arial Unicode MS"/>
-      </rPr>
-      <t>severity</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>) used during validation.</t>
-    </r>
-  </si>
-  <si>
     <t>A programming or modeling language tailored to a specific problem domain, providing constructs and abstractions closely aligned with domain concepts rather than general-purpose computation. In Freon, DSLs are designed, edited, and executed using generated tools that combine structural definitions (metamodels), projections, and validation rules.</t>
   </si>
   <si>
@@ -1305,21 +1237,12 @@
     <t>freon parse-it</t>
   </si>
   <si>
-    <t>Command that generates parser code  from .edit definition files.</t>
-  </si>
-  <si>
-    <t>Command that generates UML diagrams  from .ast definition files.</t>
-  </si>
-  <si>
     <t>freon diagram-it</t>
   </si>
   <si>
     <t>freon interpret-it</t>
   </si>
   <si>
-    <t>Command that generates interpreter code  for your language.</t>
-  </si>
-  <si>
     <t>freon clean-it</t>
   </si>
   <si>
@@ -1327,21 +1250,6 @@
   </si>
   <si>
     <t>FreProjection Interface</t>
-  </si>
-  <si>
-    <t>Interface defining  how models are parsed from text input into Freon’s AST representation.</t>
-  </si>
-  <si>
-    <t>Interface defining  the logic for resolving references and visible names within a Freon model.</t>
-  </si>
-  <si>
-    <t>Interface defining  all predefined instances and limited concepts for a given language in Freon.</t>
-  </si>
-  <si>
-    <t>Interface defining  the logic for type inference, type equality, and conformance checks.</t>
-  </si>
-  <si>
-    <t>Interface defining  how models are serialized or exported from Freon to text or files.</t>
   </si>
   <si>
     <t>FreError Interface</t>
@@ -1535,21 +1443,12 @@
     <t>Alternative namespace</t>
   </si>
   <si>
-    <t>A statement in the scoper definition that removes the names from the parent namespace, and replaces them by the names of another namespace.</t>
-  </si>
-  <si>
     <t>Box</t>
   </si>
   <si>
-    <t>Box tree / box model</t>
-  </si>
-  <si>
     <t>conformsto (keyword)</t>
   </si>
   <si>
-    <t>See Concrete Syntax Tree</t>
-  </si>
-  <si>
     <t>A user-defined replacement for, or augmentation to, the generated scoper, currently applied globally rather than per concept.</t>
   </si>
   <si>
@@ -1581,6 +1480,175 @@
   </si>
   <si>
     <t>istype (keyword)</t>
+  </si>
+  <si>
+    <t>isunique (keyword) / is-unique rule</t>
+  </si>
+  <si>
+    <t>Language engineer</t>
+  </si>
+  <si>
+    <t>Model</t>
+  </si>
+  <si>
+    <t>Named property projection</t>
+  </si>
+  <si>
+    <t>notempty (keyword) / not-empty rule</t>
+  </si>
+  <si>
+    <t>Precedence of projections</t>
+  </si>
+  <si>
+    <t>In a set of projections for the same concept, the priority of one projection over the other.</t>
+  </si>
+  <si>
+    <t>Projection set</t>
+  </si>
+  <si>
+    <t>Public property</t>
+  </si>
+  <si>
+    <t>Scope provider (or scoper)</t>
+  </si>
+  <si>
+    <t>A component that is able to determine for each term in the model which names of other elements of the model are visible.</t>
+  </si>
+  <si>
+    <t>Symbol</t>
+  </si>
+  <si>
+    <t>Term</t>
+  </si>
+  <si>
+    <t>Trigger</t>
+  </si>
+  <si>
+    <t>Type provider (or typer)</t>
+  </si>
+  <si>
+    <t>Typer</t>
+  </si>
+  <si>
+    <t>Typer file</t>
+  </si>
+  <si>
+    <t>User</t>
+  </si>
+  <si>
+    <t>Valid file</t>
+  </si>
+  <si>
+    <t>Validator</t>
+  </si>
+  <si>
+    <t>A component that is able to determine for each term in the model whether the term is correct or erroneous.</t>
+  </si>
+  <si>
+    <t>Certain behavior of the editor, for instance, the reaction to a key stroke.</t>
+  </si>
+  <si>
+    <t>Box Tree / box model</t>
+  </si>
+  <si>
+    <t>See Concrete Syntax Tree (CST).</t>
+  </si>
+  <si>
+    <t>Command that generates UML diagrams from .ast definition files.</t>
+  </si>
+  <si>
+    <t>Command that generates interpreter code for your language.</t>
+  </si>
+  <si>
+    <t>Command that generates parser code from .edit definition files.</t>
+  </si>
+  <si>
+    <t>Interface defining how models are parsed from text input into Freon’s AST representation.</t>
+  </si>
+  <si>
+    <t>Interface defining the logic for resolving references and visible names within a Freon model.</t>
+  </si>
+  <si>
+    <t>Interface defining all predefined instances and limited concepts for a given language in Freon.</t>
+  </si>
+  <si>
+    <t>Interface defining the logic for type inference, type equality, and conformance checks.</t>
+  </si>
+  <si>
+    <t>Interface defining how models are serialized or exported from Freon to text or files.</t>
+  </si>
+  <si>
+    <t>A statement in the scoper definition that removes the names from the parent namespace, and replaces them by names of another namespace.</t>
+  </si>
+  <si>
+    <t>A server implementation that stores models using the LionWeb protocol; it can be connected to Freon for model persistence.</t>
+  </si>
+  <si>
+    <t>Properties in .ast files marked with the `private` keyword; visible only within their own namespace, not when imported elsewhere.</t>
+  </si>
+  <si>
+    <t>Projectional Editor</t>
+  </si>
+  <si>
+    <t>A component that determines, for each term in the model, which type to associate with that term.</t>
+  </si>
+  <si>
+    <t>The person using Freon’s tools — e.g., the editor, scoper, or validator — to create models in a DSL.</t>
+  </si>
+  <si>
+    <t>Model Unit</t>
+  </si>
+  <si>
+    <t>Named Editor</t>
+  </si>
+  <si>
+    <t>Key editor box methods such as findParam(), setFocus(), and refreshComponent(). Used by external components and custom projections for runtime interaction with the editor.</t>
+  </si>
+  <si>
+    <t>The Freon framework for building DSL editors for the web. The name ‘Freon’ comes from the Frisian word for ‘friend’.</t>
+  </si>
+  <si>
+    <t>A predefined function in the typer, that defines that a certain type conforms to another type. The function can also be used in the validator.</t>
+  </si>
+  <si>
+    <t>A predefined function in the typer, that defines that a certain type is considered to be equal to another type. The function can also be used in the validator.</t>
+  </si>
+  <si>
+    <r>
+      <t>Definition of user-defined error messages and severity levels (</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>message</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>severity</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>) used during validation.</t>
+    </r>
   </si>
   <si>
     <r>
@@ -1589,7 +1657,6 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color theme="1"/>
         <rFont val="Arial Unicode MS"/>
       </rPr>
       <t>.valid</t>
@@ -1597,7 +1664,6 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color theme="1"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -1606,28 +1672,12 @@
     </r>
   </si>
   <si>
-    <t>isunique (keyword) / is-unique rule</t>
-  </si>
-  <si>
-    <t>Language engineer</t>
-  </si>
-  <si>
-    <t>Model</t>
-  </si>
-  <si>
-    <t>Named editor</t>
-  </si>
-  <si>
-    <t>Named property projection</t>
-  </si>
-  <si>
     <r>
       <t xml:space="preserve">Built-in validation rule ensuring that lists are not empty. Used in </t>
     </r>
     <r>
       <rPr>
         <sz val="10"/>
-        <color theme="1"/>
         <rFont val="Arial Unicode MS"/>
       </rPr>
       <t>.valid</t>
@@ -1635,7 +1685,6 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color theme="1"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -1644,37 +1693,25 @@
     </r>
   </si>
   <si>
-    <t>notempty (keyword) / not-empty rule</t>
-  </si>
-  <si>
-    <t>Precedence of projections</t>
-  </si>
-  <si>
-    <t>In a set of projections for the same concept, the priority of one projection over the other.</t>
-  </si>
-  <si>
-    <t>Projection set</t>
-  </si>
-  <si>
-    <t>Public property</t>
-  </si>
-  <si>
-    <t>Scope provider (or scoper)</t>
-  </si>
-  <si>
-    <t>A component that is able to determine for each term in the model which names of other elements of the model are visible.</t>
-  </si>
-  <si>
-    <t>Symbol</t>
-  </si>
-  <si>
-    <t>Term</t>
-  </si>
-  <si>
-    <t>Trigger</t>
-  </si>
-  <si>
-    <t>Type provider (or typer)</t>
+    <r>
+      <t>A property that is not declared </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9.9"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>private</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t> with regard to namespace imports.</t>
+    </r>
   </si>
   <si>
     <r>
@@ -1683,7 +1720,6 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color theme="1"/>
         <rFont val="Arial Unicode MS"/>
       </rPr>
       <t>FreType</t>
@@ -1691,7 +1727,6 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color theme="1"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -1700,32 +1735,17 @@
     </r>
   </si>
   <si>
-    <t>A component that is able to determine for each term in the model which type to associate with that term.</t>
-  </si>
-  <si>
-    <t>Typer</t>
-  </si>
-  <si>
-    <t>Typer file</t>
-  </si>
-  <si>
-    <t>User</t>
-  </si>
-  <si>
-    <t>Valid file</t>
-  </si>
-  <si>
-    <t>Validator</t>
-  </si>
-  <si>
-    <t>A component that is able to determine for each term in the model whether the term is correct or erroneous.</t>
+    <t>Where-clause</t>
+  </si>
+  <si>
+    <t>Valid-identifier-rule</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7">
+  <fonts count="10">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1739,11 +1759,6 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color theme="1"/>
-      <name val="Arial Unicode MS"/>
     </font>
     <font>
       <sz val="10"/>
@@ -1767,6 +1782,26 @@
     <font>
       <sz val="9.9"/>
       <color rgb="FFFF0000"/>
+      <name val="Consolas"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial Unicode MS"/>
+    </font>
+    <font>
+      <sz val="9.9"/>
       <name val="Consolas"/>
       <family val="3"/>
     </font>
@@ -1812,49 +1847,28 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2211,7 +2225,7 @@
         <v>110</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>442</v>
+        <v>424</v>
       </c>
     </row>
     <row r="7" spans="1:2">
@@ -2329,7 +2343,7 @@
         <v>106</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>443</v>
+        <v>425</v>
       </c>
     </row>
     <row r="28" spans="1:2">
@@ -2422,7 +2436,7 @@
         <v>109</v>
       </c>
       <c r="B43" s="3" t="s">
-        <v>444</v>
+        <v>426</v>
       </c>
     </row>
     <row r="44" spans="1:2">
@@ -2598,7 +2612,7 @@
         <v>113</v>
       </c>
       <c r="B72" s="6" t="s">
-        <v>445</v>
+        <v>427</v>
       </c>
     </row>
     <row r="73" spans="1:2" ht="15" thickBot="1">
@@ -2630,7 +2644,7 @@
         <v>114</v>
       </c>
       <c r="B77" s="6" t="s">
-        <v>446</v>
+        <v>428</v>
       </c>
     </row>
     <row r="78" spans="1:2" ht="15" thickBot="1">
@@ -2843,7 +2857,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DCBFF228-6AD9-43F2-8D61-560CE4700E3A}">
-  <dimension ref="A1:B256"/>
+  <dimension ref="A1:B202"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="40.33203125" style="8" customWidth="1"/>
@@ -2852,10 +2866,10 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="8" t="s">
-        <v>174</v>
+        <v>169</v>
       </c>
       <c r="B1" s="8" t="s">
-        <v>175</v>
+        <v>170</v>
       </c>
     </row>
     <row r="2" spans="1:2">
@@ -2863,47 +2877,47 @@
         <v>116</v>
       </c>
       <c r="B2" s="8" t="s">
-        <v>390</v>
+        <v>381</v>
       </c>
     </row>
     <row r="3" spans="1:2">
-      <c r="A3" s="14" t="s">
-        <v>447</v>
-      </c>
-      <c r="B3" s="9" t="s">
-        <v>38</v>
+      <c r="A3" s="8" t="s">
+        <v>429</v>
+      </c>
+      <c r="B3" s="8" t="s">
+        <v>465</v>
       </c>
     </row>
     <row r="4" spans="1:2">
-      <c r="A4" s="14" t="s">
-        <v>448</v>
-      </c>
-      <c r="B4" s="9" t="s">
-        <v>449</v>
+      <c r="A4" s="8" t="s">
+        <v>430</v>
+      </c>
+      <c r="B4" s="8" t="s">
+        <v>476</v>
       </c>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="8" t="s">
-        <v>320</v>
+        <v>312</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>321</v>
+        <v>313</v>
       </c>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="8" t="s">
-        <v>334</v>
+        <v>325</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>335</v>
+        <v>326</v>
       </c>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="8" t="s">
-        <v>214</v>
+        <v>206</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>403</v>
+        <v>393</v>
       </c>
     </row>
     <row r="8" spans="1:2">
@@ -2911,36 +2925,36 @@
         <v>49</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>391</v>
+        <v>382</v>
       </c>
     </row>
     <row r="9" spans="1:2">
-      <c r="A9" s="14" t="s">
+      <c r="A9" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="B9" s="9" t="s">
+      <c r="B9" s="8" t="s">
         <v>71</v>
       </c>
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="8" t="s">
-        <v>235</v>
+        <v>227</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>236</v>
+        <v>228</v>
       </c>
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="8" t="s">
-        <v>281</v>
+        <v>273</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>282</v>
+        <v>274</v>
       </c>
     </row>
     <row r="12" spans="1:2">
       <c r="A12" s="8" t="s">
-        <v>392</v>
+        <v>383</v>
       </c>
       <c r="B12" s="8" t="s">
         <v>117</v>
@@ -2948,1751 +2962,1527 @@
     </row>
     <row r="13" spans="1:2">
       <c r="A13" s="8" t="s">
-        <v>176</v>
+        <v>171</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>404</v>
+        <v>394</v>
       </c>
     </row>
     <row r="14" spans="1:2">
       <c r="A14" s="8" t="s">
-        <v>177</v>
+        <v>172</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>178</v>
+        <v>173</v>
       </c>
     </row>
     <row r="15" spans="1:2">
-      <c r="A15" s="14" t="s">
-        <v>450</v>
-      </c>
-      <c r="B15" s="9" t="s">
+      <c r="A15" s="8" t="s">
+        <v>431</v>
+      </c>
+      <c r="B15" s="8" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="16" spans="1:2">
       <c r="A16" s="8" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>164</v>
+        <v>484</v>
       </c>
     </row>
     <row r="17" spans="1:2">
       <c r="A17" s="8" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
     </row>
     <row r="18" spans="1:2">
       <c r="A18" s="8" t="s">
-        <v>156</v>
+        <v>152</v>
       </c>
       <c r="B18" s="8" t="s">
-        <v>393</v>
+        <v>384</v>
       </c>
     </row>
     <row r="19" spans="1:2">
       <c r="A19" s="8" t="s">
-        <v>287</v>
+        <v>466</v>
       </c>
       <c r="B19" s="8" t="s">
-        <v>288</v>
+        <v>279</v>
       </c>
     </row>
     <row r="20" spans="1:2">
-      <c r="A20" s="14" t="s">
-        <v>451</v>
-      </c>
-      <c r="B20" s="9" t="s">
-        <v>97</v>
+      <c r="A20" s="8" t="s">
+        <v>289</v>
+      </c>
+      <c r="B20" s="8" t="s">
+        <v>290</v>
       </c>
     </row>
     <row r="21" spans="1:2">
       <c r="A21" s="8" t="s">
-        <v>297</v>
+        <v>174</v>
       </c>
       <c r="B21" s="8" t="s">
-        <v>298</v>
+        <v>175</v>
       </c>
     </row>
     <row r="22" spans="1:2">
       <c r="A22" s="8" t="s">
-        <v>179</v>
+        <v>277</v>
       </c>
       <c r="B22" s="8" t="s">
-        <v>180</v>
+        <v>278</v>
       </c>
     </row>
     <row r="23" spans="1:2">
       <c r="A23" s="8" t="s">
-        <v>285</v>
+        <v>432</v>
       </c>
       <c r="B23" s="8" t="s">
-        <v>286</v>
+        <v>486</v>
       </c>
     </row>
     <row r="24" spans="1:2">
-      <c r="A24" s="14" t="s">
-        <v>452</v>
-      </c>
-      <c r="B24" s="9" t="s">
-        <v>45</v>
+      <c r="A24" s="8" t="s">
+        <v>310</v>
+      </c>
+      <c r="B24" s="8" t="s">
+        <v>311</v>
       </c>
     </row>
     <row r="25" spans="1:2">
       <c r="A25" s="8" t="s">
-        <v>318</v>
+        <v>20</v>
       </c>
       <c r="B25" s="8" t="s">
-        <v>319</v>
+        <v>467</v>
       </c>
     </row>
     <row r="26" spans="1:2">
-      <c r="A26" s="14" t="s">
-        <v>20</v>
-      </c>
-      <c r="B26" s="9" t="s">
-        <v>453</v>
+      <c r="A26" s="8" t="s">
+        <v>147</v>
+      </c>
+      <c r="B26" s="8" t="s">
+        <v>148</v>
       </c>
     </row>
     <row r="27" spans="1:2">
       <c r="A27" s="8" t="s">
-        <v>151</v>
+        <v>343</v>
       </c>
       <c r="B27" s="8" t="s">
-        <v>152</v>
+        <v>344</v>
       </c>
     </row>
     <row r="28" spans="1:2">
       <c r="A28" s="8" t="s">
-        <v>352</v>
+        <v>218</v>
       </c>
       <c r="B28" s="8" t="s">
-        <v>353</v>
+        <v>488</v>
       </c>
     </row>
     <row r="29" spans="1:2">
       <c r="A29" s="8" t="s">
-        <v>226</v>
+        <v>145</v>
       </c>
       <c r="B29" s="8" t="s">
-        <v>394</v>
+        <v>146</v>
       </c>
     </row>
     <row r="30" spans="1:2">
       <c r="A30" s="8" t="s">
-        <v>149</v>
+        <v>161</v>
       </c>
       <c r="B30" s="8" t="s">
-        <v>150</v>
+        <v>433</v>
       </c>
     </row>
     <row r="31" spans="1:2">
       <c r="A31" s="8" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="B31" s="8" t="s">
-        <v>454</v>
+        <v>434</v>
       </c>
     </row>
     <row r="32" spans="1:2">
       <c r="A32" s="8" t="s">
-        <v>168</v>
+        <v>141</v>
       </c>
       <c r="B32" s="8" t="s">
-        <v>455</v>
+        <v>142</v>
       </c>
     </row>
     <row r="33" spans="1:2">
       <c r="A33" s="8" t="s">
-        <v>145</v>
+        <v>314</v>
       </c>
       <c r="B33" s="8" t="s">
-        <v>146</v>
+        <v>435</v>
       </c>
     </row>
     <row r="34" spans="1:2">
       <c r="A34" s="8" t="s">
-        <v>322</v>
+        <v>219</v>
       </c>
       <c r="B34" s="8" t="s">
-        <v>456</v>
+        <v>220</v>
       </c>
     </row>
     <row r="35" spans="1:2">
       <c r="A35" s="8" t="s">
-        <v>227</v>
+        <v>283</v>
       </c>
       <c r="B35" s="8" t="s">
-        <v>228</v>
+        <v>284</v>
       </c>
     </row>
     <row r="36" spans="1:2">
       <c r="A36" s="8" t="s">
-        <v>291</v>
+        <v>386</v>
       </c>
       <c r="B36" s="8" t="s">
-        <v>292</v>
+        <v>385</v>
       </c>
     </row>
     <row r="37" spans="1:2">
       <c r="A37" s="8" t="s">
-        <v>396</v>
+        <v>267</v>
       </c>
       <c r="B37" s="8" t="s">
-        <v>395</v>
+        <v>268</v>
       </c>
     </row>
     <row r="38" spans="1:2">
       <c r="A38" s="8" t="s">
-        <v>275</v>
+        <v>387</v>
       </c>
       <c r="B38" s="8" t="s">
-        <v>276</v>
+        <v>388</v>
       </c>
     </row>
     <row r="39" spans="1:2">
       <c r="A39" s="8" t="s">
-        <v>397</v>
+        <v>30</v>
       </c>
       <c r="B39" s="8" t="s">
-        <v>398</v>
+        <v>98</v>
       </c>
     </row>
     <row r="40" spans="1:2">
-      <c r="A40" s="14" t="s">
-        <v>30</v>
-      </c>
-      <c r="B40" s="9" t="s">
-        <v>98</v>
+      <c r="A40" s="8" t="s">
+        <v>437</v>
+      </c>
+      <c r="B40" s="8" t="s">
+        <v>67</v>
       </c>
     </row>
     <row r="41" spans="1:2">
-      <c r="A41" s="14" t="s">
-        <v>458</v>
-      </c>
-      <c r="B41" s="9" t="s">
-        <v>67</v>
+      <c r="A41" s="8" t="s">
+        <v>176</v>
+      </c>
+      <c r="B41" s="8" t="s">
+        <v>436</v>
       </c>
     </row>
     <row r="42" spans="1:2">
       <c r="A42" s="8" t="s">
-        <v>181</v>
+        <v>285</v>
       </c>
       <c r="B42" s="8" t="s">
-        <v>457</v>
+        <v>286</v>
       </c>
     </row>
     <row r="43" spans="1:2">
       <c r="A43" s="8" t="s">
-        <v>293</v>
+        <v>118</v>
       </c>
       <c r="B43" s="8" t="s">
-        <v>294</v>
+        <v>119</v>
       </c>
     </row>
     <row r="44" spans="1:2">
       <c r="A44" s="8" t="s">
-        <v>118</v>
+        <v>438</v>
       </c>
       <c r="B44" s="8" t="s">
-        <v>119</v>
+        <v>65</v>
       </c>
     </row>
     <row r="45" spans="1:2">
-      <c r="A45" s="14" t="s">
-        <v>459</v>
-      </c>
-      <c r="B45" s="9" t="s">
-        <v>65</v>
+      <c r="A45" s="8" t="s">
+        <v>439</v>
+      </c>
+      <c r="B45" s="8" t="s">
+        <v>487</v>
       </c>
     </row>
     <row r="46" spans="1:2">
-      <c r="A46" s="14" t="s">
-        <v>460</v>
-      </c>
-      <c r="B46" s="9" t="s">
-        <v>55</v>
+      <c r="A46" s="8" t="s">
+        <v>365</v>
+      </c>
+      <c r="B46" s="8" t="s">
+        <v>366</v>
       </c>
     </row>
     <row r="47" spans="1:2">
       <c r="A47" s="8" t="s">
-        <v>374</v>
+        <v>238</v>
       </c>
       <c r="B47" s="8" t="s">
-        <v>375</v>
+        <v>239</v>
       </c>
     </row>
     <row r="48" spans="1:2">
       <c r="A48" s="8" t="s">
-        <v>246</v>
+        <v>240</v>
       </c>
       <c r="B48" s="8" t="s">
-        <v>247</v>
+        <v>241</v>
       </c>
     </row>
     <row r="49" spans="1:2">
       <c r="A49" s="8" t="s">
-        <v>248</v>
+        <v>271</v>
       </c>
       <c r="B49" s="8" t="s">
-        <v>249</v>
+        <v>272</v>
       </c>
     </row>
     <row r="50" spans="1:2">
       <c r="A50" s="8" t="s">
-        <v>279</v>
+        <v>440</v>
       </c>
       <c r="B50" s="8" t="s">
-        <v>280</v>
+        <v>395</v>
       </c>
     </row>
     <row r="51" spans="1:2">
       <c r="A51" s="8" t="s">
-        <v>461</v>
+        <v>153</v>
       </c>
       <c r="B51" s="8" t="s">
-        <v>405</v>
+        <v>154</v>
       </c>
     </row>
     <row r="52" spans="1:2">
       <c r="A52" s="8" t="s">
-        <v>157</v>
+        <v>441</v>
       </c>
       <c r="B52" s="8" t="s">
-        <v>158</v>
+        <v>61</v>
       </c>
     </row>
     <row r="53" spans="1:2">
-      <c r="A53" s="14" t="s">
-        <v>462</v>
-      </c>
-      <c r="B53" s="9" t="s">
-        <v>61</v>
+      <c r="A53" s="8" t="s">
+        <v>294</v>
+      </c>
+      <c r="B53" s="8" t="s">
+        <v>295</v>
       </c>
     </row>
     <row r="54" spans="1:2">
       <c r="A54" s="8" t="s">
-        <v>302</v>
+        <v>298</v>
       </c>
       <c r="B54" s="8" t="s">
-        <v>303</v>
+        <v>299</v>
       </c>
     </row>
     <row r="55" spans="1:2">
       <c r="A55" s="8" t="s">
-        <v>306</v>
+        <v>302</v>
       </c>
       <c r="B55" s="8" t="s">
-        <v>307</v>
+        <v>303</v>
       </c>
     </row>
     <row r="56" spans="1:2">
       <c r="A56" s="8" t="s">
-        <v>310</v>
+        <v>157</v>
       </c>
       <c r="B56" s="8" t="s">
-        <v>311</v>
+        <v>158</v>
       </c>
     </row>
     <row r="57" spans="1:2">
       <c r="A57" s="8" t="s">
-        <v>161</v>
+        <v>296</v>
       </c>
       <c r="B57" s="8" t="s">
-        <v>162</v>
+        <v>297</v>
       </c>
     </row>
     <row r="58" spans="1:2">
       <c r="A58" s="8" t="s">
-        <v>304</v>
+        <v>300</v>
       </c>
       <c r="B58" s="8" t="s">
-        <v>305</v>
+        <v>301</v>
       </c>
     </row>
     <row r="59" spans="1:2">
       <c r="A59" s="8" t="s">
-        <v>308</v>
+        <v>346</v>
       </c>
       <c r="B59" s="8" t="s">
-        <v>309</v>
+        <v>347</v>
       </c>
     </row>
     <row r="60" spans="1:2">
       <c r="A60" s="8" t="s">
-        <v>355</v>
+        <v>408</v>
       </c>
       <c r="B60" s="8" t="s">
-        <v>356</v>
+        <v>409</v>
       </c>
     </row>
     <row r="61" spans="1:2">
       <c r="A61" s="8" t="s">
-        <v>426</v>
+        <v>410</v>
       </c>
       <c r="B61" s="8" t="s">
-        <v>427</v>
+        <v>342</v>
       </c>
     </row>
     <row r="62" spans="1:2">
       <c r="A62" s="8" t="s">
-        <v>428</v>
+        <v>411</v>
       </c>
       <c r="B62" s="8" t="s">
-        <v>351</v>
+        <v>413</v>
       </c>
     </row>
     <row r="63" spans="1:2">
       <c r="A63" s="8" t="s">
-        <v>429</v>
+        <v>412</v>
       </c>
       <c r="B63" s="8" t="s">
-        <v>431</v>
+        <v>293</v>
       </c>
     </row>
     <row r="64" spans="1:2">
       <c r="A64" s="8" t="s">
-        <v>430</v>
+        <v>120</v>
       </c>
       <c r="B64" s="8" t="s">
-        <v>301</v>
+        <v>121</v>
       </c>
     </row>
     <row r="65" spans="1:2">
       <c r="A65" s="8" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="B65" s="8" t="s">
-        <v>121</v>
+        <v>485</v>
       </c>
     </row>
     <row r="66" spans="1:2">
       <c r="A66" s="8" t="s">
-        <v>122</v>
+        <v>225</v>
       </c>
       <c r="B66" s="8" t="s">
-        <v>123</v>
+        <v>389</v>
       </c>
     </row>
     <row r="67" spans="1:2">
       <c r="A67" s="8" t="s">
-        <v>233</v>
+        <v>401</v>
       </c>
       <c r="B67" s="8" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
     </row>
     <row r="68" spans="1:2">
       <c r="A68" s="8" t="s">
-        <v>411</v>
+        <v>405</v>
       </c>
       <c r="B68" s="8" t="s">
-        <v>410</v>
+        <v>406</v>
       </c>
     </row>
     <row r="69" spans="1:2">
       <c r="A69" s="8" t="s">
-        <v>418</v>
+        <v>403</v>
       </c>
       <c r="B69" s="8" t="s">
-        <v>419</v>
+        <v>468</v>
       </c>
     </row>
     <row r="70" spans="1:2">
       <c r="A70" s="8" t="s">
-        <v>415</v>
+        <v>398</v>
       </c>
       <c r="B70" s="8" t="s">
-        <v>414</v>
+        <v>399</v>
       </c>
     </row>
     <row r="71" spans="1:2">
       <c r="A71" s="8" t="s">
-        <v>408</v>
+        <v>226</v>
       </c>
       <c r="B71" s="8" t="s">
-        <v>409</v>
+        <v>414</v>
       </c>
     </row>
     <row r="72" spans="1:2">
       <c r="A72" s="8" t="s">
-        <v>234</v>
+        <v>123</v>
       </c>
       <c r="B72" s="8" t="s">
-        <v>432</v>
+        <v>124</v>
       </c>
     </row>
     <row r="73" spans="1:2">
       <c r="A73" s="8" t="s">
-        <v>124</v>
+        <v>404</v>
       </c>
       <c r="B73" s="8" t="s">
-        <v>125</v>
+        <v>469</v>
       </c>
     </row>
     <row r="74" spans="1:2">
       <c r="A74" s="8" t="s">
-        <v>416</v>
+        <v>291</v>
       </c>
       <c r="B74" s="8" t="s">
-        <v>417</v>
+        <v>292</v>
       </c>
     </row>
     <row r="75" spans="1:2">
       <c r="A75" s="8" t="s">
-        <v>299</v>
+        <v>402</v>
       </c>
       <c r="B75" s="8" t="s">
-        <v>300</v>
+        <v>470</v>
       </c>
     </row>
     <row r="76" spans="1:2">
       <c r="A76" s="8" t="s">
-        <v>412</v>
+        <v>396</v>
       </c>
       <c r="B76" s="8" t="s">
-        <v>413</v>
+        <v>397</v>
       </c>
     </row>
     <row r="77" spans="1:2">
       <c r="A77" s="8" t="s">
-        <v>406</v>
+        <v>223</v>
       </c>
       <c r="B77" s="8" t="s">
-        <v>407</v>
+        <v>390</v>
       </c>
     </row>
     <row r="78" spans="1:2">
       <c r="A78" s="8" t="s">
-        <v>231</v>
+        <v>224</v>
       </c>
       <c r="B78" s="8" t="s">
-        <v>400</v>
+        <v>391</v>
       </c>
     </row>
     <row r="79" spans="1:2">
       <c r="A79" s="8" t="s">
-        <v>232</v>
+        <v>304</v>
       </c>
       <c r="B79" s="8" t="s">
-        <v>401</v>
+        <v>305</v>
       </c>
     </row>
     <row r="80" spans="1:2">
       <c r="A80" s="8" t="s">
-        <v>312</v>
+        <v>407</v>
       </c>
       <c r="B80" s="8" t="s">
-        <v>313</v>
+        <v>341</v>
       </c>
     </row>
     <row r="81" spans="1:2">
       <c r="A81" s="8" t="s">
-        <v>420</v>
+        <v>151</v>
       </c>
       <c r="B81" s="8" t="s">
-        <v>350</v>
+        <v>415</v>
       </c>
     </row>
     <row r="82" spans="1:2">
       <c r="A82" s="8" t="s">
-        <v>155</v>
+        <v>353</v>
       </c>
       <c r="B82" s="8" t="s">
-        <v>433</v>
+        <v>354</v>
       </c>
     </row>
     <row r="83" spans="1:2">
       <c r="A83" s="8" t="s">
-        <v>362</v>
+        <v>164</v>
       </c>
       <c r="B83" s="8" t="s">
-        <v>363</v>
+        <v>471</v>
       </c>
     </row>
     <row r="84" spans="1:2">
       <c r="A84" s="8" t="s">
-        <v>169</v>
+        <v>348</v>
       </c>
       <c r="B84" s="8" t="s">
-        <v>421</v>
+        <v>416</v>
       </c>
     </row>
     <row r="85" spans="1:2">
       <c r="A85" s="8" t="s">
-        <v>357</v>
+        <v>160</v>
       </c>
       <c r="B85" s="8" t="s">
-        <v>434</v>
+        <v>472</v>
       </c>
     </row>
     <row r="86" spans="1:2">
       <c r="A86" s="8" t="s">
-        <v>165</v>
+        <v>357</v>
       </c>
       <c r="B86" s="8" t="s">
-        <v>422</v>
+        <v>417</v>
       </c>
     </row>
     <row r="87" spans="1:2">
       <c r="A87" s="8" t="s">
-        <v>366</v>
+        <v>166</v>
       </c>
       <c r="B87" s="8" t="s">
-        <v>435</v>
+        <v>473</v>
       </c>
     </row>
     <row r="88" spans="1:2">
       <c r="A88" s="8" t="s">
-        <v>171</v>
+        <v>137</v>
       </c>
       <c r="B88" s="8" t="s">
-        <v>423</v>
+        <v>138</v>
       </c>
     </row>
     <row r="89" spans="1:2">
       <c r="A89" s="8" t="s">
-        <v>141</v>
+        <v>306</v>
       </c>
       <c r="B89" s="8" t="s">
-        <v>142</v>
+        <v>307</v>
       </c>
     </row>
     <row r="90" spans="1:2">
       <c r="A90" s="8" t="s">
-        <v>314</v>
+        <v>308</v>
       </c>
       <c r="B90" s="8" t="s">
-        <v>315</v>
+        <v>309</v>
       </c>
     </row>
     <row r="91" spans="1:2">
       <c r="A91" s="8" t="s">
-        <v>316</v>
+        <v>205</v>
       </c>
       <c r="B91" s="8" t="s">
-        <v>317</v>
+        <v>418</v>
       </c>
     </row>
     <row r="92" spans="1:2">
       <c r="A92" s="8" t="s">
-        <v>213</v>
+        <v>350</v>
       </c>
       <c r="B92" s="8" t="s">
-        <v>436</v>
+        <v>419</v>
       </c>
     </row>
     <row r="93" spans="1:2">
       <c r="A93" s="8" t="s">
-        <v>359</v>
+        <v>162</v>
       </c>
       <c r="B93" s="8" t="s">
-        <v>437</v>
+        <v>474</v>
       </c>
     </row>
     <row r="94" spans="1:2">
       <c r="A94" s="8" t="s">
-        <v>167</v>
+        <v>351</v>
       </c>
       <c r="B94" s="8" t="s">
-        <v>424</v>
+        <v>352</v>
       </c>
     </row>
     <row r="95" spans="1:2">
       <c r="A95" s="8" t="s">
-        <v>360</v>
+        <v>231</v>
       </c>
       <c r="B95" s="8" t="s">
-        <v>361</v>
+        <v>232</v>
       </c>
     </row>
     <row r="96" spans="1:2">
       <c r="A96" s="8" t="s">
-        <v>239</v>
+        <v>349</v>
       </c>
       <c r="B96" s="8" t="s">
-        <v>240</v>
+        <v>420</v>
       </c>
     </row>
     <row r="97" spans="1:2">
       <c r="A97" s="8" t="s">
-        <v>358</v>
+        <v>421</v>
       </c>
       <c r="B97" s="8" t="s">
-        <v>438</v>
+        <v>422</v>
       </c>
     </row>
     <row r="98" spans="1:2">
       <c r="A98" s="8" t="s">
-        <v>439</v>
+        <v>355</v>
       </c>
       <c r="B98" s="8" t="s">
-        <v>440</v>
+        <v>356</v>
       </c>
     </row>
     <row r="99" spans="1:2">
       <c r="A99" s="8" t="s">
-        <v>364</v>
+        <v>165</v>
       </c>
       <c r="B99" s="8" t="s">
-        <v>365</v>
+        <v>475</v>
       </c>
     </row>
     <row r="100" spans="1:2">
       <c r="A100" s="8" t="s">
-        <v>170</v>
+        <v>423</v>
       </c>
       <c r="B100" s="8" t="s">
-        <v>425</v>
+        <v>392</v>
       </c>
     </row>
     <row r="101" spans="1:2">
       <c r="A101" s="8" t="s">
-        <v>441</v>
+        <v>177</v>
       </c>
       <c r="B101" s="8" t="s">
-        <v>402</v>
+        <v>178</v>
       </c>
     </row>
     <row r="102" spans="1:2">
       <c r="A102" s="8" t="s">
-        <v>182</v>
+        <v>200</v>
       </c>
       <c r="B102" s="8" t="s">
-        <v>183</v>
+        <v>201</v>
       </c>
     </row>
     <row r="103" spans="1:2">
       <c r="A103" s="8" t="s">
-        <v>209</v>
+        <v>335</v>
       </c>
       <c r="B103" s="8" t="s">
-        <v>210</v>
+        <v>336</v>
       </c>
     </row>
     <row r="104" spans="1:2">
       <c r="A104" s="8" t="s">
-        <v>344</v>
+        <v>315</v>
       </c>
       <c r="B104" s="8" t="s">
-        <v>345</v>
+        <v>316</v>
       </c>
     </row>
     <row r="105" spans="1:2">
       <c r="A105" s="8" t="s">
-        <v>323</v>
+        <v>327</v>
       </c>
       <c r="B105" s="8" t="s">
-        <v>324</v>
+        <v>328</v>
       </c>
     </row>
     <row r="106" spans="1:2">
       <c r="A106" s="8" t="s">
-        <v>336</v>
+        <v>202</v>
       </c>
       <c r="B106" s="8" t="s">
-        <v>337</v>
+        <v>203</v>
       </c>
     </row>
     <row r="107" spans="1:2">
       <c r="A107" s="8" t="s">
-        <v>211</v>
+        <v>233</v>
       </c>
       <c r="B107" s="8" t="s">
-        <v>212</v>
+        <v>234</v>
       </c>
     </row>
     <row r="108" spans="1:2">
       <c r="A108" s="8" t="s">
-        <v>241</v>
+        <v>237</v>
       </c>
       <c r="B108" s="8" t="s">
-        <v>242</v>
+        <v>442</v>
       </c>
     </row>
     <row r="109" spans="1:2">
       <c r="A109" s="8" t="s">
-        <v>245</v>
+        <v>242</v>
       </c>
       <c r="B109" s="8" t="s">
-        <v>463</v>
+        <v>243</v>
       </c>
     </row>
     <row r="110" spans="1:2">
       <c r="A110" s="8" t="s">
-        <v>250</v>
+        <v>235</v>
       </c>
       <c r="B110" s="8" t="s">
-        <v>251</v>
+        <v>236</v>
       </c>
     </row>
     <row r="111" spans="1:2">
       <c r="A111" s="8" t="s">
-        <v>243</v>
+        <v>329</v>
       </c>
       <c r="B111" s="8" t="s">
-        <v>244</v>
+        <v>330</v>
       </c>
     </row>
     <row r="112" spans="1:2">
       <c r="A112" s="8" t="s">
-        <v>338</v>
+        <v>443</v>
       </c>
       <c r="B112" s="8" t="s">
-        <v>339</v>
+        <v>199</v>
       </c>
     </row>
     <row r="113" spans="1:2">
       <c r="A113" s="8" t="s">
-        <v>464</v>
+        <v>444</v>
       </c>
       <c r="B113" s="8" t="s">
-        <v>208</v>
+        <v>489</v>
       </c>
     </row>
     <row r="114" spans="1:2">
       <c r="A114" s="8" t="s">
-        <v>466</v>
-      </c>
-      <c r="B114" t="s">
-        <v>465</v>
+        <v>445</v>
+      </c>
+      <c r="B114" s="8" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="115" spans="1:2">
-      <c r="A115" s="14" t="s">
-        <v>467</v>
-      </c>
-      <c r="B115" s="9" t="s">
-        <v>101</v>
+      <c r="A115" s="8" t="s">
+        <v>358</v>
+      </c>
+      <c r="B115" s="8" t="s">
+        <v>359</v>
       </c>
     </row>
     <row r="116" spans="1:2">
       <c r="A116" s="8" t="s">
-        <v>367</v>
+        <v>204</v>
       </c>
       <c r="B116" s="8" t="s">
-        <v>368</v>
+        <v>63</v>
       </c>
     </row>
     <row r="117" spans="1:2">
       <c r="A117" s="8" t="s">
-        <v>184</v>
-      </c>
-      <c r="B117" s="12" t="s">
-        <v>63</v>
+        <v>125</v>
+      </c>
+      <c r="B117" s="8" t="s">
+        <v>126</v>
       </c>
     </row>
     <row r="118" spans="1:2">
       <c r="A118" s="8" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B118" s="8" t="s">
-        <v>127</v>
+        <v>477</v>
       </c>
     </row>
     <row r="119" spans="1:2">
       <c r="A119" s="8" t="s">
-        <v>128</v>
+        <v>250</v>
       </c>
       <c r="B119" s="8" t="s">
-        <v>129</v>
+        <v>251</v>
       </c>
     </row>
     <row r="120" spans="1:2">
       <c r="A120" s="8" t="s">
-        <v>258</v>
+        <v>248</v>
       </c>
       <c r="B120" s="8" t="s">
-        <v>259</v>
+        <v>249</v>
       </c>
     </row>
     <row r="121" spans="1:2">
       <c r="A121" s="8" t="s">
-        <v>256</v>
+        <v>246</v>
       </c>
       <c r="B121" s="8" t="s">
-        <v>257</v>
+        <v>247</v>
       </c>
     </row>
     <row r="122" spans="1:2">
       <c r="A122" s="8" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="B122" s="8" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
     </row>
     <row r="123" spans="1:2">
       <c r="A123" s="8" t="s">
-        <v>260</v>
+        <v>179</v>
       </c>
       <c r="B123" s="8" t="s">
-        <v>261</v>
+        <v>180</v>
       </c>
     </row>
     <row r="124" spans="1:2">
       <c r="A124" s="8" t="s">
-        <v>185</v>
+        <v>229</v>
       </c>
       <c r="B124" s="8" t="s">
-        <v>186</v>
+        <v>230</v>
       </c>
     </row>
     <row r="125" spans="1:2">
       <c r="A125" s="8" t="s">
-        <v>237</v>
+        <v>446</v>
       </c>
       <c r="B125" s="8" t="s">
-        <v>238</v>
+        <v>41</v>
       </c>
     </row>
     <row r="126" spans="1:2">
-      <c r="A126" s="15" t="s">
-        <v>468</v>
-      </c>
-      <c r="B126" s="12" t="s">
-        <v>41</v>
+      <c r="A126" s="8" t="s">
+        <v>482</v>
+      </c>
+      <c r="B126" s="8" t="s">
+        <v>128</v>
       </c>
     </row>
     <row r="127" spans="1:2">
       <c r="A127" s="8" t="s">
-        <v>130</v>
+        <v>362</v>
       </c>
       <c r="B127" s="8" t="s">
-        <v>131</v>
+        <v>363</v>
       </c>
     </row>
     <row r="128" spans="1:2">
       <c r="A128" s="8" t="s">
-        <v>371</v>
+        <v>129</v>
       </c>
       <c r="B128" s="8" t="s">
-        <v>372</v>
+        <v>130</v>
       </c>
     </row>
     <row r="129" spans="1:2">
       <c r="A129" s="8" t="s">
-        <v>132</v>
+        <v>483</v>
       </c>
       <c r="B129" s="8" t="s">
-        <v>133</v>
+        <v>74</v>
       </c>
     </row>
     <row r="130" spans="1:2">
-      <c r="A130" s="15" t="s">
-        <v>469</v>
-      </c>
-      <c r="B130" s="12" t="s">
-        <v>74</v>
+      <c r="A130" s="8" t="s">
+        <v>379</v>
+      </c>
+      <c r="B130" s="8" t="s">
+        <v>380</v>
       </c>
     </row>
     <row r="131" spans="1:2">
       <c r="A131" s="8" t="s">
-        <v>388</v>
+        <v>447</v>
       </c>
       <c r="B131" s="8" t="s">
-        <v>389</v>
+        <v>75</v>
       </c>
     </row>
     <row r="132" spans="1:2">
-      <c r="A132" s="15" t="s">
-        <v>470</v>
-      </c>
-      <c r="B132" s="12" t="s">
-        <v>75</v>
+      <c r="A132" s="8" t="s">
+        <v>317</v>
+      </c>
+      <c r="B132" s="8" t="s">
+        <v>104</v>
       </c>
     </row>
     <row r="133" spans="1:2">
       <c r="A133" s="8" t="s">
-        <v>325</v>
-      </c>
-      <c r="B133" s="12" t="s">
-        <v>104</v>
+        <v>181</v>
+      </c>
+      <c r="B133" s="8" t="s">
+        <v>182</v>
       </c>
     </row>
     <row r="134" spans="1:2">
       <c r="A134" s="8" t="s">
-        <v>187</v>
+        <v>318</v>
       </c>
       <c r="B134" s="8" t="s">
-        <v>188</v>
+        <v>319</v>
       </c>
     </row>
     <row r="135" spans="1:2">
       <c r="A135" s="8" t="s">
-        <v>326</v>
+        <v>448</v>
       </c>
       <c r="B135" s="8" t="s">
-        <v>327</v>
+        <v>490</v>
       </c>
     </row>
     <row r="136" spans="1:2">
       <c r="A136" s="8" t="s">
-        <v>472</v>
-      </c>
-      <c r="B136" t="s">
-        <v>471</v>
+        <v>131</v>
+      </c>
+      <c r="B136" s="8" t="s">
+        <v>132</v>
       </c>
     </row>
     <row r="137" spans="1:2">
       <c r="A137" s="8" t="s">
-        <v>134</v>
+        <v>254</v>
       </c>
       <c r="B137" s="8" t="s">
-        <v>135</v>
+        <v>345</v>
       </c>
     </row>
     <row r="138" spans="1:2">
       <c r="A138" s="8" t="s">
-        <v>262</v>
+        <v>337</v>
       </c>
       <c r="B138" s="8" t="s">
-        <v>354</v>
+        <v>338</v>
       </c>
     </row>
     <row r="139" spans="1:2">
       <c r="A139" s="8" t="s">
-        <v>346</v>
+        <v>269</v>
       </c>
       <c r="B139" s="8" t="s">
-        <v>347</v>
+        <v>270</v>
       </c>
     </row>
     <row r="140" spans="1:2">
       <c r="A140" s="8" t="s">
-        <v>277</v>
+        <v>320</v>
       </c>
       <c r="B140" s="8" t="s">
-        <v>278</v>
+        <v>321</v>
       </c>
     </row>
     <row r="141" spans="1:2">
       <c r="A141" s="8" t="s">
-        <v>328</v>
+        <v>133</v>
       </c>
       <c r="B141" s="8" t="s">
-        <v>329</v>
+        <v>115</v>
       </c>
     </row>
     <row r="142" spans="1:2">
       <c r="A142" s="8" t="s">
-        <v>136</v>
+        <v>373</v>
       </c>
       <c r="B142" s="8" t="s">
-        <v>115</v>
+        <v>374</v>
       </c>
     </row>
     <row r="143" spans="1:2">
       <c r="A143" s="8" t="s">
-        <v>382</v>
+        <v>275</v>
       </c>
       <c r="B143" s="8" t="s">
-        <v>383</v>
+        <v>276</v>
       </c>
     </row>
     <row r="144" spans="1:2">
       <c r="A144" s="8" t="s">
-        <v>283</v>
+        <v>449</v>
       </c>
       <c r="B144" s="8" t="s">
-        <v>284</v>
+        <v>450</v>
       </c>
     </row>
     <row r="145" spans="1:2">
-      <c r="A145" s="15" t="s">
-        <v>473</v>
-      </c>
-      <c r="B145" s="12" t="s">
-        <v>474</v>
+      <c r="A145" s="8" t="s">
+        <v>331</v>
+      </c>
+      <c r="B145" s="8" t="s">
+        <v>332</v>
       </c>
     </row>
     <row r="146" spans="1:2">
       <c r="A146" s="8" t="s">
-        <v>340</v>
+        <v>322</v>
       </c>
       <c r="B146" s="8" t="s">
-        <v>341</v>
+        <v>478</v>
       </c>
     </row>
     <row r="147" spans="1:2">
       <c r="A147" s="8" t="s">
-        <v>330</v>
+        <v>134</v>
       </c>
       <c r="B147" s="8" t="s">
-        <v>331</v>
+        <v>135</v>
       </c>
     </row>
     <row r="148" spans="1:2">
       <c r="A148" s="8" t="s">
-        <v>137</v>
+        <v>149</v>
       </c>
       <c r="B148" s="8" t="s">
-        <v>138</v>
+        <v>150</v>
       </c>
     </row>
     <row r="149" spans="1:2">
       <c r="A149" s="8" t="s">
-        <v>153</v>
+        <v>451</v>
       </c>
       <c r="B149" s="8" t="s">
-        <v>154</v>
+        <v>68</v>
       </c>
     </row>
     <row r="150" spans="1:2">
-      <c r="A150" s="15" t="s">
-        <v>475</v>
-      </c>
-      <c r="B150" s="12" t="s">
-        <v>68</v>
+      <c r="A150" s="8" t="s">
+        <v>280</v>
+      </c>
+      <c r="B150" s="8" t="s">
+        <v>136</v>
       </c>
     </row>
     <row r="151" spans="1:2">
       <c r="A151" s="8" t="s">
-        <v>139</v>
+        <v>479</v>
       </c>
       <c r="B151" s="8" t="s">
-        <v>140</v>
+        <v>183</v>
       </c>
     </row>
     <row r="152" spans="1:2">
       <c r="A152" s="8" t="s">
-        <v>189</v>
+        <v>452</v>
       </c>
       <c r="B152" s="8" t="s">
-        <v>190</v>
+        <v>491</v>
       </c>
     </row>
     <row r="153" spans="1:2">
-      <c r="A153" s="15" t="s">
-        <v>476</v>
-      </c>
-      <c r="B153" s="12" t="s">
-        <v>446</v>
+      <c r="A153" s="8" t="s">
+        <v>184</v>
+      </c>
+      <c r="B153" s="8" t="s">
+        <v>185</v>
       </c>
     </row>
     <row r="154" spans="1:2">
       <c r="A154" s="8" t="s">
-        <v>191</v>
+        <v>186</v>
       </c>
       <c r="B154" s="8" t="s">
-        <v>192</v>
+        <v>187</v>
       </c>
     </row>
     <row r="155" spans="1:2">
       <c r="A155" s="8" t="s">
-        <v>193</v>
+        <v>155</v>
       </c>
       <c r="B155" s="8" t="s">
-        <v>194</v>
+        <v>156</v>
       </c>
     </row>
     <row r="156" spans="1:2">
       <c r="A156" s="8" t="s">
-        <v>159</v>
+        <v>263</v>
       </c>
       <c r="B156" s="8" t="s">
-        <v>160</v>
+        <v>264</v>
       </c>
     </row>
     <row r="157" spans="1:2">
       <c r="A157" s="8" t="s">
-        <v>271</v>
+        <v>261</v>
       </c>
       <c r="B157" s="8" t="s">
-        <v>272</v>
+        <v>262</v>
       </c>
     </row>
     <row r="158" spans="1:2">
       <c r="A158" s="8" t="s">
-        <v>269</v>
+        <v>265</v>
       </c>
       <c r="B158" s="8" t="s">
-        <v>270</v>
+        <v>266</v>
       </c>
     </row>
     <row r="159" spans="1:2">
       <c r="A159" s="8" t="s">
-        <v>273</v>
+        <v>257</v>
       </c>
       <c r="B159" s="8" t="s">
-        <v>274</v>
+        <v>258</v>
       </c>
     </row>
     <row r="160" spans="1:2">
       <c r="A160" s="8" t="s">
-        <v>265</v>
+        <v>259</v>
       </c>
       <c r="B160" s="8" t="s">
-        <v>266</v>
+        <v>260</v>
       </c>
     </row>
     <row r="161" spans="1:2">
       <c r="A161" s="8" t="s">
-        <v>267</v>
+        <v>244</v>
       </c>
       <c r="B161" s="8" t="s">
-        <v>268</v>
+        <v>245</v>
       </c>
     </row>
     <row r="162" spans="1:2">
       <c r="A162" s="8" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
       <c r="B162" s="8" t="s">
-        <v>253</v>
+        <v>256</v>
       </c>
     </row>
     <row r="163" spans="1:2">
       <c r="A163" s="8" t="s">
-        <v>263</v>
+        <v>188</v>
       </c>
       <c r="B163" s="8" t="s">
-        <v>264</v>
+        <v>189</v>
       </c>
     </row>
     <row r="164" spans="1:2">
       <c r="A164" s="8" t="s">
-        <v>195</v>
+        <v>453</v>
       </c>
       <c r="B164" s="8" t="s">
-        <v>196</v>
+        <v>454</v>
       </c>
     </row>
     <row r="165" spans="1:2">
-      <c r="A165" s="15" t="s">
-        <v>477</v>
-      </c>
-      <c r="B165" s="12" t="s">
-        <v>478</v>
+      <c r="A165" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="B165" s="8" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="166" spans="1:2">
-      <c r="A166" s="15" t="s">
-        <v>25</v>
-      </c>
-      <c r="B166" s="12" t="s">
-        <v>47</v>
+      <c r="A166" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="B166" s="8" t="s">
+        <v>72</v>
       </c>
     </row>
     <row r="167" spans="1:2">
-      <c r="A167" s="15" t="s">
-        <v>33</v>
-      </c>
-      <c r="B167" s="12" t="s">
-        <v>72</v>
+      <c r="A167" s="8" t="s">
+        <v>190</v>
+      </c>
+      <c r="B167" s="8" t="s">
+        <v>191</v>
       </c>
     </row>
     <row r="168" spans="1:2">
       <c r="A168" s="8" t="s">
-        <v>197</v>
+        <v>360</v>
       </c>
       <c r="B168" s="8" t="s">
-        <v>198</v>
+        <v>361</v>
       </c>
     </row>
     <row r="169" spans="1:2">
       <c r="A169" s="8" t="s">
-        <v>369</v>
+        <v>196</v>
       </c>
       <c r="B169" s="8" t="s">
-        <v>370</v>
+        <v>197</v>
       </c>
     </row>
     <row r="170" spans="1:2">
       <c r="A170" s="8" t="s">
-        <v>203</v>
+        <v>333</v>
       </c>
       <c r="B170" s="8" t="s">
-        <v>204</v>
+        <v>334</v>
       </c>
     </row>
     <row r="171" spans="1:2">
       <c r="A171" s="8" t="s">
-        <v>342</v>
+        <v>221</v>
       </c>
       <c r="B171" s="8" t="s">
-        <v>343</v>
+        <v>222</v>
       </c>
     </row>
     <row r="172" spans="1:2">
       <c r="A172" s="8" t="s">
-        <v>229</v>
+        <v>212</v>
       </c>
       <c r="B172" s="8" t="s">
-        <v>230</v>
+        <v>213</v>
       </c>
     </row>
     <row r="173" spans="1:2">
       <c r="A173" s="8" t="s">
-        <v>220</v>
+        <v>167</v>
       </c>
       <c r="B173" s="8" t="s">
-        <v>221</v>
+        <v>168</v>
       </c>
     </row>
     <row r="174" spans="1:2">
       <c r="A174" s="8" t="s">
-        <v>172</v>
+        <v>139</v>
       </c>
       <c r="B174" s="8" t="s">
-        <v>173</v>
+        <v>140</v>
       </c>
     </row>
     <row r="175" spans="1:2">
       <c r="A175" s="8" t="s">
-        <v>143</v>
+        <v>377</v>
       </c>
       <c r="B175" s="8" t="s">
-        <v>144</v>
+        <v>378</v>
       </c>
     </row>
     <row r="176" spans="1:2">
       <c r="A176" s="8" t="s">
-        <v>386</v>
+        <v>281</v>
       </c>
       <c r="B176" s="8" t="s">
-        <v>387</v>
+        <v>282</v>
       </c>
     </row>
     <row r="177" spans="1:2">
       <c r="A177" s="8" t="s">
-        <v>289</v>
+        <v>455</v>
       </c>
       <c r="B177" s="8" t="s">
-        <v>290</v>
+        <v>89</v>
       </c>
     </row>
     <row r="178" spans="1:2">
-      <c r="A178" s="15" t="s">
-        <v>479</v>
-      </c>
-      <c r="B178" s="12" t="s">
-        <v>89</v>
+      <c r="A178" s="8" t="s">
+        <v>456</v>
+      </c>
+      <c r="B178" s="8" t="s">
+        <v>82</v>
       </c>
     </row>
     <row r="179" spans="1:2">
-      <c r="A179" s="15" t="s">
-        <v>480</v>
-      </c>
-      <c r="B179" s="12" t="s">
-        <v>82</v>
+      <c r="A179" s="8" t="s">
+        <v>457</v>
+      </c>
+      <c r="B179" s="8" t="s">
+        <v>90</v>
       </c>
     </row>
     <row r="180" spans="1:2">
-      <c r="A180" s="15" t="s">
-        <v>481</v>
-      </c>
-      <c r="B180" s="12" t="s">
-        <v>90</v>
+      <c r="A180" s="8" t="s">
+        <v>287</v>
+      </c>
+      <c r="B180" s="8" t="s">
+        <v>288</v>
       </c>
     </row>
     <row r="181" spans="1:2">
       <c r="A181" s="8" t="s">
-        <v>295</v>
+        <v>216</v>
       </c>
       <c r="B181" s="8" t="s">
-        <v>296</v>
+        <v>217</v>
       </c>
     </row>
     <row r="182" spans="1:2">
       <c r="A182" s="8" t="s">
-        <v>224</v>
+        <v>207</v>
       </c>
       <c r="B182" s="8" t="s">
-        <v>225</v>
+        <v>208</v>
       </c>
     </row>
     <row r="183" spans="1:2">
       <c r="A183" s="8" t="s">
-        <v>215</v>
+        <v>198</v>
       </c>
       <c r="B183" s="8" t="s">
-        <v>216</v>
+        <v>492</v>
       </c>
     </row>
     <row r="184" spans="1:2">
       <c r="A184" s="8" t="s">
-        <v>207</v>
-      </c>
-      <c r="B184" t="s">
-        <v>483</v>
+        <v>371</v>
+      </c>
+      <c r="B184" s="8" t="s">
+        <v>372</v>
       </c>
     </row>
     <row r="185" spans="1:2">
       <c r="A185" s="8" t="s">
-        <v>380</v>
+        <v>369</v>
       </c>
       <c r="B185" s="8" t="s">
-        <v>381</v>
+        <v>370</v>
       </c>
     </row>
     <row r="186" spans="1:2">
       <c r="A186" s="8" t="s">
-        <v>378</v>
+        <v>367</v>
       </c>
       <c r="B186" s="8" t="s">
-        <v>379</v>
+        <v>368</v>
       </c>
     </row>
     <row r="187" spans="1:2">
       <c r="A187" s="8" t="s">
-        <v>376</v>
+        <v>458</v>
       </c>
       <c r="B187" s="8" t="s">
-        <v>377</v>
+        <v>480</v>
       </c>
     </row>
     <row r="188" spans="1:2">
-      <c r="A188" s="15" t="s">
-        <v>482</v>
-      </c>
-      <c r="B188" s="12" t="s">
-        <v>484</v>
+      <c r="A188" s="8" t="s">
+        <v>339</v>
+      </c>
+      <c r="B188" s="8" t="s">
+        <v>340</v>
       </c>
     </row>
     <row r="189" spans="1:2">
       <c r="A189" s="8" t="s">
-        <v>205</v>
+        <v>459</v>
       </c>
       <c r="B189" s="8" t="s">
-        <v>206</v>
+        <v>48</v>
       </c>
     </row>
     <row r="190" spans="1:2">
       <c r="A190" s="8" t="s">
-        <v>348</v>
+        <v>460</v>
       </c>
       <c r="B190" s="8" t="s">
-        <v>349</v>
+        <v>73</v>
       </c>
     </row>
     <row r="191" spans="1:2">
-      <c r="A191" s="15" t="s">
-        <v>485</v>
-      </c>
-      <c r="B191" s="12" t="s">
-        <v>48</v>
+      <c r="A191" s="8" t="s">
+        <v>192</v>
+      </c>
+      <c r="B191" s="8" t="s">
+        <v>193</v>
       </c>
     </row>
     <row r="192" spans="1:2">
-      <c r="A192" s="15" t="s">
-        <v>486</v>
-      </c>
-      <c r="B192" s="12" t="s">
-        <v>73</v>
+      <c r="A192" s="8" t="s">
+        <v>375</v>
+      </c>
+      <c r="B192" s="8" t="s">
+        <v>376</v>
       </c>
     </row>
     <row r="193" spans="1:2">
       <c r="A193" s="8" t="s">
-        <v>199</v>
+        <v>461</v>
       </c>
       <c r="B193" s="8" t="s">
-        <v>200</v>
+        <v>481</v>
       </c>
     </row>
     <row r="194" spans="1:2">
       <c r="A194" s="8" t="s">
-        <v>384</v>
+        <v>462</v>
       </c>
       <c r="B194" s="8" t="s">
-        <v>385</v>
+        <v>105</v>
       </c>
     </row>
     <row r="195" spans="1:2">
-      <c r="A195" s="15" t="s">
-        <v>487</v>
-      </c>
-      <c r="B195" s="12" t="s">
-        <v>60</v>
+      <c r="A195" s="8" t="s">
+        <v>214</v>
+      </c>
+      <c r="B195" s="8" t="s">
+        <v>215</v>
       </c>
     </row>
     <row r="196" spans="1:2">
-      <c r="A196" s="15" t="s">
-        <v>488</v>
-      </c>
-      <c r="B196" s="12" t="s">
-        <v>105</v>
+      <c r="A196" s="8" t="s">
+        <v>194</v>
+      </c>
+      <c r="B196" s="8" t="s">
+        <v>195</v>
       </c>
     </row>
     <row r="197" spans="1:2">
-      <c r="A197" s="17" t="s">
-        <v>222</v>
-      </c>
-      <c r="B197" s="17" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="198" spans="1:2" ht="15" thickBot="1">
-      <c r="A198" s="17" t="s">
-        <v>201</v>
-      </c>
-      <c r="B198" s="17" t="s">
-        <v>202</v>
-      </c>
-    </row>
-    <row r="199" spans="1:2" ht="15" thickBot="1">
-      <c r="A199" s="13" t="s">
-        <v>219</v>
-      </c>
-      <c r="B199" s="13" t="s">
-        <v>373</v>
-      </c>
-    </row>
-    <row r="200" spans="1:2" ht="15" thickBot="1">
-      <c r="A200" s="16" t="s">
-        <v>489</v>
-      </c>
-      <c r="B200" s="11" t="s">
-        <v>490</v>
-      </c>
-    </row>
-    <row r="201" spans="1:2" ht="15" thickBot="1">
-      <c r="A201" s="13" t="s">
-        <v>217</v>
-      </c>
-      <c r="B201" s="13" t="s">
-        <v>218</v>
-      </c>
-    </row>
-    <row r="202" spans="1:2" ht="15" thickBot="1">
-      <c r="A202" s="16" t="s">
-        <v>13</v>
-      </c>
-      <c r="B202" s="11" t="s">
+      <c r="A197" s="8" t="s">
+        <v>211</v>
+      </c>
+      <c r="B197" s="8" t="s">
+        <v>364</v>
+      </c>
+    </row>
+    <row r="198" spans="1:2">
+      <c r="A198" s="8" t="s">
+        <v>463</v>
+      </c>
+      <c r="B198" s="8" t="s">
+        <v>464</v>
+      </c>
+    </row>
+    <row r="199" spans="1:2">
+      <c r="A199" s="8" t="s">
+        <v>209</v>
+      </c>
+      <c r="B199" s="8" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="200" spans="1:2">
+      <c r="A200" s="8" t="s">
+        <v>494</v>
+      </c>
+      <c r="B200" s="8" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="203" spans="1:2" ht="15" thickBot="1">
-      <c r="A203" s="13" t="s">
-        <v>332</v>
-      </c>
-      <c r="B203" s="13" t="s">
-        <v>333</v>
-      </c>
-    </row>
-    <row r="204" spans="1:2" ht="15" thickBot="1">
-      <c r="A204" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="B204" s="11" t="s">
+    <row r="201" spans="1:2">
+      <c r="A201" s="8" t="s">
+        <v>323</v>
+      </c>
+      <c r="B201" s="8" t="s">
+        <v>324</v>
+      </c>
+    </row>
+    <row r="202" spans="1:2">
+      <c r="A202" s="8" t="s">
+        <v>493</v>
+      </c>
+      <c r="B202" s="8" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="205" spans="1:2" ht="15" thickBot="1">
-      <c r="A205" s="16"/>
-      <c r="B205" s="11"/>
-    </row>
-    <row r="206" spans="1:2" ht="15" thickBot="1">
-      <c r="A206" s="16"/>
-      <c r="B206" s="11"/>
-    </row>
-    <row r="207" spans="1:2" ht="15" thickBot="1">
-      <c r="A207" s="13"/>
-      <c r="B207" s="13"/>
-    </row>
-    <row r="208" spans="1:2" ht="15" thickBot="1">
-      <c r="A208" s="4"/>
-      <c r="B208" s="10"/>
-    </row>
-    <row r="209" spans="1:2" ht="15" thickBot="1">
-      <c r="A209" s="4"/>
-      <c r="B209" s="10"/>
-    </row>
-    <row r="210" spans="1:2" ht="15" thickBot="1">
-      <c r="A210" s="4"/>
-      <c r="B210" s="10"/>
-    </row>
-    <row r="211" spans="1:2" ht="15" thickBot="1">
-      <c r="A211" s="4"/>
-      <c r="B211" s="10"/>
-    </row>
-    <row r="212" spans="1:2" ht="15" thickBot="1">
-      <c r="A212" s="4"/>
-      <c r="B212" s="10"/>
-    </row>
-    <row r="213" spans="1:2" ht="15" thickBot="1">
-      <c r="A213" s="4"/>
-      <c r="B213" s="10"/>
-    </row>
-    <row r="214" spans="1:2" ht="15" thickBot="1">
-      <c r="A214" s="4"/>
-      <c r="B214" s="10"/>
-    </row>
-    <row r="215" spans="1:2" ht="15" thickBot="1">
-      <c r="A215" s="4"/>
-      <c r="B215" s="10"/>
-    </row>
-    <row r="216" spans="1:2" ht="15" thickBot="1">
-      <c r="A216" s="4"/>
-      <c r="B216" s="10"/>
-    </row>
-    <row r="217" spans="1:2" ht="15" thickBot="1">
-      <c r="A217" s="4"/>
-      <c r="B217" s="10"/>
-    </row>
-    <row r="218" spans="1:2" ht="15" thickBot="1">
-      <c r="A218" s="4"/>
-      <c r="B218" s="10"/>
-    </row>
-    <row r="219" spans="1:2" ht="15" thickBot="1">
-      <c r="A219" s="4"/>
-      <c r="B219" s="10"/>
-    </row>
-    <row r="220" spans="1:2" ht="15" thickBot="1">
-      <c r="A220" s="4"/>
-      <c r="B220" s="10"/>
-    </row>
-    <row r="221" spans="1:2" ht="15" thickBot="1">
-      <c r="A221" s="4"/>
-      <c r="B221" s="10"/>
-    </row>
-    <row r="222" spans="1:2" ht="15" thickBot="1">
-      <c r="A222" s="4"/>
-      <c r="B222" s="10"/>
-    </row>
-    <row r="223" spans="1:2" ht="15" thickBot="1">
-      <c r="A223" s="4"/>
-      <c r="B223" s="10"/>
-    </row>
-    <row r="224" spans="1:2" ht="15" thickBot="1">
-      <c r="A224" s="4"/>
-      <c r="B224" s="10"/>
-    </row>
-    <row r="225" spans="1:2" ht="15" thickBot="1">
-      <c r="A225" s="4"/>
-      <c r="B225" s="10"/>
-    </row>
-    <row r="226" spans="1:2" ht="15" thickBot="1">
-      <c r="A226" s="4"/>
-      <c r="B226" s="10"/>
-    </row>
-    <row r="227" spans="1:2" ht="15" thickBot="1">
-      <c r="A227" s="4"/>
-      <c r="B227" s="10"/>
-    </row>
-    <row r="228" spans="1:2" ht="15" thickBot="1">
-      <c r="A228" s="4"/>
-      <c r="B228" s="10"/>
-    </row>
-    <row r="229" spans="1:2" ht="15" thickBot="1">
-      <c r="A229" s="4"/>
-      <c r="B229" s="10"/>
-    </row>
-    <row r="230" spans="1:2" ht="15" thickBot="1">
-      <c r="A230" s="4"/>
-      <c r="B230" s="10"/>
-    </row>
-    <row r="231" spans="1:2" ht="15" thickBot="1">
-      <c r="A231" s="4"/>
-      <c r="B231" s="10"/>
-    </row>
-    <row r="232" spans="1:2" ht="15" thickBot="1">
-      <c r="A232" s="4"/>
-      <c r="B232" s="10"/>
-    </row>
-    <row r="233" spans="1:2" ht="15" thickBot="1">
-      <c r="A233" s="4"/>
-      <c r="B233" s="10"/>
-    </row>
-    <row r="234" spans="1:2" ht="15" thickBot="1">
-      <c r="A234" s="4"/>
-      <c r="B234" s="10"/>
-    </row>
-    <row r="235" spans="1:2" ht="15" thickBot="1">
-      <c r="A235" s="4"/>
-      <c r="B235" s="10"/>
-    </row>
-    <row r="236" spans="1:2" ht="15" thickBot="1">
-      <c r="A236" s="4"/>
-      <c r="B236" s="10"/>
-    </row>
-    <row r="237" spans="1:2" ht="15" thickBot="1">
-      <c r="A237" s="4"/>
-      <c r="B237" s="10"/>
-    </row>
-    <row r="238" spans="1:2" ht="15" thickBot="1">
-      <c r="A238" s="4"/>
-      <c r="B238" s="10"/>
-    </row>
-    <row r="239" spans="1:2" ht="15" thickBot="1">
-      <c r="A239" s="4"/>
-      <c r="B239" s="10"/>
-    </row>
-    <row r="240" spans="1:2" ht="15" thickBot="1">
-      <c r="A240" s="4"/>
-      <c r="B240" s="10"/>
-    </row>
-    <row r="241" spans="1:2" ht="15" thickBot="1">
-      <c r="A241" s="4"/>
-      <c r="B241" s="10"/>
-    </row>
-    <row r="242" spans="1:2" ht="15" thickBot="1">
-      <c r="A242" s="4"/>
-      <c r="B242" s="10"/>
-    </row>
-    <row r="243" spans="1:2" ht="15" thickBot="1">
-      <c r="A243" s="4"/>
-      <c r="B243" s="10"/>
-    </row>
-    <row r="244" spans="1:2" ht="15" thickBot="1">
-      <c r="A244" s="4"/>
-      <c r="B244" s="10"/>
-    </row>
-    <row r="245" spans="1:2" ht="15" thickBot="1">
-      <c r="A245" s="4"/>
-      <c r="B245" s="10"/>
-    </row>
-    <row r="246" spans="1:2" ht="15" thickBot="1">
-      <c r="A246" s="4"/>
-      <c r="B246" s="10"/>
-    </row>
-    <row r="247" spans="1:2" ht="15" thickBot="1">
-      <c r="A247" s="4"/>
-      <c r="B247" s="10"/>
-    </row>
-    <row r="248" spans="1:2" ht="15" thickBot="1">
-      <c r="A248" s="4"/>
-      <c r="B248" s="10"/>
-    </row>
-    <row r="249" spans="1:2" ht="15" thickBot="1">
-      <c r="A249" s="4"/>
-      <c r="B249" s="10"/>
-    </row>
-    <row r="250" spans="1:2" ht="15" thickBot="1">
-      <c r="A250" s="4"/>
-      <c r="B250" s="10"/>
-    </row>
-    <row r="251" spans="1:2" ht="15" thickBot="1">
-      <c r="A251" s="4"/>
-      <c r="B251" s="10"/>
-    </row>
-    <row r="252" spans="1:2" ht="15" thickBot="1">
-      <c r="A252" s="4"/>
-      <c r="B252" s="10"/>
-    </row>
-    <row r="253" spans="1:2" ht="15" thickBot="1">
-      <c r="A253" s="4"/>
-      <c r="B253" s="10"/>
-    </row>
-    <row r="254" spans="1:2" ht="15" thickBot="1">
-      <c r="A254" s="4"/>
-      <c r="B254" s="10"/>
-    </row>
-    <row r="255" spans="1:2" ht="15" thickBot="1">
-      <c r="A255" s="4"/>
-      <c r="B255" s="10"/>
-    </row>
-    <row r="256" spans="1:2" ht="15" thickBot="1">
-      <c r="A256" s="4"/>
-      <c r="B256" s="10"/>
-    </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A1:B257">
-    <sortCondition ref="A211:A257"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A1:B255">
+    <sortCondition ref="A209:A255"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>